<commit_message>
Standard Format: Arial 10
</commit_message>
<xml_diff>
--- a/src/v2/tests/header_test.xlsx
+++ b/src/v2/tests/header_test.xlsx
@@ -1368,7 +1368,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm-dd-yy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1378,25 +1378,28 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1599,35 +1602,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1637,14 +1640,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1653,10 +1656,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2108,18 +2112,12 @@
         <f>D8</f>
         <v>0</v>
       </c>
-      <c r="E9" s="10">
-        <f>E8</f>
-        <v>0</v>
-      </c>
+      <c r="E9" s="10"/>
       <c r="F9" s="23">
         <f>F8</f>
         <v>0</v>
       </c>
-      <c r="G9" s="10">
-        <f>G8</f>
-        <v>0</v>
-      </c>
+      <c r="G9" s="10"/>
       <c r="H9" s="10"/>
       <c r="J9" s="13"/>
     </row>
@@ -2262,1697 +2260,1697 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:63">
-      <c r="A1" t="s">
+      <c r="A1" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BC1" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BD1" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BE1" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BF1" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BG1" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BH1" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BI1" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BJ1" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BK1" s="25" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:63">
-      <c r="A2" t="s">
+      <c r="A2" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="V2" t="s">
+      <c r="V2" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="X2" t="s">
+      <c r="X2" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Y2" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="Z2" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AA2" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AB2" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AC2" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AD2" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AE2" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AF2" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AG2" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AH2" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AI2" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AJ2" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AK2" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AL2" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AM2" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AN2" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AO2" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AP2" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AQ2" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AR2" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AS2" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AT2" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AU2" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AV2" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AW2" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="AX2" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="AY2" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="AZ2" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BA2" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BB2" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BC2" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BD2" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BE2" s="25" t="s">
         <v>118</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BF2" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BG2" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BH2" s="25" t="s">
         <v>121</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BI2" s="25" t="s">
         <v>122</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BJ2" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BK2" s="25" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:63">
-      <c r="A3" t="s">
+      <c r="A3" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="T3" t="s">
+      <c r="T3" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="U3" t="s">
+      <c r="U3" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="V3" t="s">
+      <c r="V3" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="X3" t="s">
+      <c r="X3" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Y3" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="Z3" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AA3" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AB3" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AC3" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AD3" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="AE3" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AF3" s="25" t="s">
         <v>154</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AG3" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="AH3" t="s">
+      <c r="AH3" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="AI3" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="AJ3" t="s">
+      <c r="AJ3" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="AK3" t="s">
+      <c r="AK3" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="AL3" t="s">
+      <c r="AL3" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="AM3" t="s">
+      <c r="AM3" s="25" t="s">
         <v>161</v>
       </c>
-      <c r="AN3" t="s">
+      <c r="AN3" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="AO3" t="s">
+      <c r="AO3" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="AP3" t="s">
+      <c r="AP3" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="AQ3" t="s">
+      <c r="AQ3" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="AR3" t="s">
+      <c r="AR3" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="AS3" t="s">
+      <c r="AS3" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="AT3" t="s">
+      <c r="AT3" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="AU3" t="s">
+      <c r="AU3" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="AV3" t="s">
+      <c r="AV3" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="AW3" t="s">
+      <c r="AW3" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="AX3" t="s">
+      <c r="AX3" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="AY3" t="s">
+      <c r="AY3" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="AZ3" t="s">
+      <c r="AZ3" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="BA3" t="s">
+      <c r="BA3" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="BB3" t="s">
+      <c r="BB3" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="BC3" t="s">
+      <c r="BC3" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="BD3" t="s">
+      <c r="BD3" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="BE3" t="s">
+      <c r="BE3" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="BF3" t="s">
+      <c r="BF3" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="BG3" t="s">
+      <c r="BG3" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="BH3" t="s">
+      <c r="BH3" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="BI3" t="s">
+      <c r="BI3" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="BJ3" t="s">
+      <c r="BJ3" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="BK3" t="s">
+      <c r="BK3" s="25" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:63">
-      <c r="A4" t="s">
+      <c r="A4" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="25" t="s">
         <v>185</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="25" t="s">
         <v>187</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="25" t="s">
         <v>195</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="R4" t="s">
+      <c r="R4" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="S4" t="s">
+      <c r="S4" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="T4" t="s">
+      <c r="T4" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="U4" t="s">
+      <c r="U4" s="25" t="s">
         <v>203</v>
       </c>
-      <c r="V4" t="s">
+      <c r="V4" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="W4" t="s">
+      <c r="W4" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="X4" t="s">
+      <c r="X4" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Y4" s="25" t="s">
         <v>206</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="Z4" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AA4" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="AB4" t="s">
+      <c r="AB4" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AC4" s="25" t="s">
         <v>210</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AD4" s="25" t="s">
         <v>211</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AE4" s="25" t="s">
         <v>212</v>
       </c>
-      <c r="AF4" t="s">
+      <c r="AF4" s="25" t="s">
         <v>213</v>
       </c>
-      <c r="AG4" t="s">
+      <c r="AG4" s="25" t="s">
         <v>214</v>
       </c>
-      <c r="AH4" t="s">
+      <c r="AH4" s="25" t="s">
         <v>215</v>
       </c>
-      <c r="AI4" t="s">
+      <c r="AI4" s="25" t="s">
         <v>216</v>
       </c>
-      <c r="AJ4" t="s">
+      <c r="AJ4" s="25" t="s">
         <v>217</v>
       </c>
-      <c r="AK4" t="s">
+      <c r="AK4" s="25" t="s">
         <v>218</v>
       </c>
-      <c r="AL4" t="s">
+      <c r="AL4" s="25" t="s">
         <v>219</v>
       </c>
-      <c r="AM4" t="s">
+      <c r="AM4" s="25" t="s">
         <v>220</v>
       </c>
-      <c r="AN4" t="s">
+      <c r="AN4" s="25" t="s">
         <v>221</v>
       </c>
-      <c r="AO4" t="s">
+      <c r="AO4" s="25" t="s">
         <v>222</v>
       </c>
-      <c r="AP4" t="s">
+      <c r="AP4" s="25" t="s">
         <v>223</v>
       </c>
-      <c r="AQ4" t="s">
+      <c r="AQ4" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="AR4" t="s">
+      <c r="AR4" s="25" t="s">
         <v>224</v>
       </c>
-      <c r="AS4" t="s">
+      <c r="AS4" s="25" t="s">
         <v>225</v>
       </c>
-      <c r="AT4" t="s">
+      <c r="AT4" s="25" t="s">
         <v>226</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AU4" s="25" t="s">
         <v>227</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AV4" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="AW4" t="s">
+      <c r="AW4" s="25" t="s">
         <v>229</v>
       </c>
-      <c r="AX4" t="s">
+      <c r="AX4" s="25" t="s">
         <v>230</v>
       </c>
-      <c r="AY4" t="s">
+      <c r="AY4" s="25" t="s">
         <v>231</v>
       </c>
-      <c r="AZ4" t="s">
+      <c r="AZ4" s="25" t="s">
         <v>232</v>
       </c>
-      <c r="BA4" t="s">
+      <c r="BA4" s="25" t="s">
         <v>233</v>
       </c>
-      <c r="BB4" t="s">
+      <c r="BB4" s="25" t="s">
         <v>234</v>
       </c>
-      <c r="BC4" t="s">
+      <c r="BC4" s="25" t="s">
         <v>235</v>
       </c>
-      <c r="BD4" t="s">
+      <c r="BD4" s="25" t="s">
         <v>236</v>
       </c>
-      <c r="BE4" t="s">
+      <c r="BE4" s="25" t="s">
         <v>237</v>
       </c>
-      <c r="BF4" t="s">
+      <c r="BF4" s="25" t="s">
         <v>238</v>
       </c>
-      <c r="BG4" t="s">
+      <c r="BG4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="BH4" t="s">
+      <c r="BH4" s="25" t="s">
         <v>239</v>
       </c>
-      <c r="BI4" t="s">
+      <c r="BI4" s="25" t="s">
         <v>240</v>
       </c>
-      <c r="BJ4" t="s">
+      <c r="BJ4" s="25" t="s">
         <v>241</v>
       </c>
-      <c r="BK4" t="s">
+      <c r="BK4" s="25" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:63">
-      <c r="A5" t="s">
+      <c r="A5" s="25" t="s">
         <v>243</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="25" t="s">
         <v>244</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="25" t="s">
         <v>245</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="25" t="s">
         <v>246</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="25" t="s">
         <v>247</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="25" t="s">
         <v>248</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="25" t="s">
         <v>249</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="25" t="s">
         <v>250</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="25" t="s">
         <v>251</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="25" t="s">
         <v>252</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="25" t="s">
         <v>253</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="25" t="s">
         <v>254</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="O5" t="s">
+      <c r="O5" s="25" t="s">
         <v>256</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P5" s="25" t="s">
         <v>257</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="Q5" s="25" t="s">
         <v>258</v>
       </c>
-      <c r="R5" t="s">
+      <c r="R5" s="25" t="s">
         <v>259</v>
       </c>
-      <c r="S5" t="s">
+      <c r="S5" s="25" t="s">
         <v>260</v>
       </c>
-      <c r="T5" t="s">
+      <c r="T5" s="25" t="s">
         <v>261</v>
       </c>
-      <c r="U5" t="s">
+      <c r="U5" s="25" t="s">
         <v>262</v>
       </c>
-      <c r="V5" t="s">
+      <c r="V5" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="W5" t="s">
+      <c r="W5" s="25" t="s">
         <v>263</v>
       </c>
-      <c r="X5" t="s">
+      <c r="X5" s="25" t="s">
         <v>264</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Y5" s="25" t="s">
         <v>265</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="Z5" s="25" t="s">
         <v>266</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AA5" s="25" t="s">
         <v>267</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="AB5" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AC5" s="25" t="s">
         <v>268</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AD5" s="25" t="s">
         <v>269</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AE5" s="25" t="s">
         <v>270</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AF5" s="25" t="s">
         <v>271</v>
       </c>
-      <c r="AG5" t="s">
+      <c r="AG5" s="25" t="s">
         <v>272</v>
       </c>
-      <c r="AH5" t="s">
+      <c r="AH5" s="25" t="s">
         <v>273</v>
       </c>
-      <c r="AI5" t="s">
+      <c r="AI5" s="25" t="s">
         <v>274</v>
       </c>
-      <c r="AJ5" t="s">
+      <c r="AJ5" s="25" t="s">
         <v>275</v>
       </c>
-      <c r="AK5" t="s">
+      <c r="AK5" s="25" t="s">
         <v>276</v>
       </c>
-      <c r="AL5" t="s">
+      <c r="AL5" s="25" t="s">
         <v>277</v>
       </c>
-      <c r="AM5" t="s">
+      <c r="AM5" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="AN5" t="s">
+      <c r="AN5" s="25" t="s">
         <v>279</v>
       </c>
-      <c r="AO5" t="s">
+      <c r="AO5" s="25" t="s">
         <v>280</v>
       </c>
-      <c r="AP5" t="s">
+      <c r="AP5" s="25" t="s">
         <v>281</v>
       </c>
-      <c r="AQ5" t="s">
+      <c r="AQ5" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="AR5" t="s">
+      <c r="AR5" s="25" t="s">
         <v>282</v>
       </c>
-      <c r="AS5" t="s">
+      <c r="AS5" s="25" t="s">
         <v>283</v>
       </c>
-      <c r="AT5" t="s">
+      <c r="AT5" s="25" t="s">
         <v>284</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AU5" s="25" t="s">
         <v>285</v>
       </c>
-      <c r="AV5" t="s">
+      <c r="AV5" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="AW5" t="s">
+      <c r="AW5" s="25" t="s">
         <v>286</v>
       </c>
-      <c r="AX5" t="s">
+      <c r="AX5" s="25" t="s">
         <v>287</v>
       </c>
-      <c r="AY5" t="s">
+      <c r="AY5" s="25" t="s">
         <v>288</v>
       </c>
-      <c r="AZ5" t="s">
+      <c r="AZ5" s="25" t="s">
         <v>289</v>
       </c>
-      <c r="BA5" t="s">
+      <c r="BA5" s="25" t="s">
         <v>290</v>
       </c>
-      <c r="BB5" t="s">
+      <c r="BB5" s="25" t="s">
         <v>291</v>
       </c>
-      <c r="BC5" t="s">
+      <c r="BC5" s="25" t="s">
         <v>292</v>
       </c>
-      <c r="BD5" t="s">
+      <c r="BD5" s="25" t="s">
         <v>293</v>
       </c>
-      <c r="BE5" t="s">
+      <c r="BE5" s="25" t="s">
         <v>294</v>
       </c>
-      <c r="BF5" t="s">
+      <c r="BF5" s="25" t="s">
         <v>295</v>
       </c>
-      <c r="BG5" t="s">
+      <c r="BG5" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="BH5" t="s">
+      <c r="BH5" s="25" t="s">
         <v>296</v>
       </c>
-      <c r="BI5" t="s">
+      <c r="BI5" s="25" t="s">
         <v>297</v>
       </c>
-      <c r="BJ5" t="s">
+      <c r="BJ5" s="25" t="s">
         <v>298</v>
       </c>
-      <c r="BK5" t="s">
+      <c r="BK5" s="25" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="6" spans="1:63">
-      <c r="A6" t="s">
+      <c r="A6" s="25" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:63">
-      <c r="A7" t="s">
+      <c r="A7" s="25" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:63">
-      <c r="A8" t="s">
+      <c r="A8" s="25" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="9" spans="1:63">
-      <c r="A9" t="s">
+      <c r="A9" s="25" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="10" spans="1:63">
-      <c r="A10" t="s">
+      <c r="A10" s="25" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="11" spans="1:63">
-      <c r="A11" t="s">
+      <c r="A11" s="25" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="12" spans="1:63">
-      <c r="A12" t="s">
+      <c r="A12" s="25" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:63">
-      <c r="A13" t="s">
+      <c r="A13" s="25" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="14" spans="1:63">
-      <c r="A14" t="s">
+      <c r="A14" s="25" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="15" spans="1:63">
-      <c r="A15" t="s">
+      <c r="A15" s="25" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:63">
-      <c r="A16" t="s">
+      <c r="A16" s="25" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" t="s">
+      <c r="A17" s="25" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" t="s">
+      <c r="A18" s="25" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" t="s">
+      <c r="A19" s="25" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" t="s">
+      <c r="A20" s="25" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" t="s">
+      <c r="A21" s="25" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" t="s">
+      <c r="A22" s="25" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" t="s">
+      <c r="A23" s="25" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" t="s">
+      <c r="A24" s="25" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="25" spans="1:1">
-      <c r="A25" t="s">
+      <c r="A25" s="25" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="26" spans="1:1">
-      <c r="A26" t="s">
+      <c r="A26" s="25" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="27" spans="1:1">
-      <c r="A27" t="s">
+      <c r="A27" s="25" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="28" spans="1:1">
-      <c r="A28" t="s">
+      <c r="A28" s="25" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" t="s">
+      <c r="A29" s="25" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="30" spans="1:1">
-      <c r="A30" t="s">
+      <c r="A30" s="25" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" t="s">
+      <c r="A31" s="25" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" t="s">
+      <c r="A32" s="25" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" t="s">
+      <c r="A33" s="25" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" t="s">
+      <c r="A34" s="25" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" t="s">
+      <c r="A35" s="25" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" t="s">
+      <c r="A36" s="25" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="37" spans="1:1">
-      <c r="A37" t="s">
+      <c r="A37" s="25" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" t="s">
+      <c r="A38" s="25" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" t="s">
+      <c r="A39" s="25" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="40" spans="1:1">
-      <c r="A40" t="s">
+      <c r="A40" s="25" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="41" spans="1:1">
-      <c r="A41" t="s">
+      <c r="A41" s="25" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" t="s">
+      <c r="A42" s="25" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="43" spans="1:1">
-      <c r="A43" t="s">
+      <c r="A43" s="25" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="44" spans="1:1">
-      <c r="A44" t="s">
+      <c r="A44" s="25" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="45" spans="1:1">
-      <c r="A45" t="s">
+      <c r="A45" s="25" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="46" spans="1:1">
-      <c r="A46" t="s">
+      <c r="A46" s="25" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="47" spans="1:1">
-      <c r="A47" t="s">
+      <c r="A47" s="25" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" t="s">
+      <c r="A48" s="25" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" t="s">
+      <c r="A49" s="25" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" t="s">
+      <c r="A50" s="25" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" t="s">
+      <c r="A51" s="25" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="52" spans="1:1">
-      <c r="A52" t="s">
+      <c r="A52" s="25" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="53" spans="1:1">
-      <c r="A53" t="s">
+      <c r="A53" s="25" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="54" spans="1:1">
-      <c r="A54" t="s">
+      <c r="A54" s="25" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" t="s">
+      <c r="A55" s="25" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="56" spans="1:1">
-      <c r="A56" t="s">
+      <c r="A56" s="25" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="57" spans="1:1">
-      <c r="A57" t="s">
+      <c r="A57" s="25" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="58" spans="1:1">
-      <c r="A58" t="s">
+      <c r="A58" s="25" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="59" spans="1:1">
-      <c r="A59" t="s">
+      <c r="A59" s="25" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="60" spans="1:1">
-      <c r="A60" t="s">
+      <c r="A60" s="25" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="61" spans="1:1">
-      <c r="A61" t="s">
+      <c r="A61" s="25" t="s">
         <v>355</v>
       </c>
     </row>
     <row r="62" spans="1:1">
-      <c r="A62" t="s">
+      <c r="A62" s="25" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="63" spans="1:1">
-      <c r="A63" t="s">
+      <c r="A63" s="25" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="64" spans="1:1">
-      <c r="A64" t="s">
+      <c r="A64" s="25" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="65" spans="1:1">
-      <c r="A65" t="s">
+      <c r="A65" s="25" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="66" spans="1:1">
-      <c r="A66" t="s">
+      <c r="A66" s="25" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="67" spans="1:1">
-      <c r="A67" t="s">
+      <c r="A67" s="25" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="68" spans="1:1">
-      <c r="A68" t="s">
+      <c r="A68" s="25" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="69" spans="1:1">
-      <c r="A69" t="s">
+      <c r="A69" s="25" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="70" spans="1:1">
-      <c r="A70" t="s">
+      <c r="A70" s="25" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="71" spans="1:1">
-      <c r="A71" t="s">
+      <c r="A71" s="25" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="72" spans="1:1">
-      <c r="A72" t="s">
+      <c r="A72" s="25" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="73" spans="1:1">
-      <c r="A73" t="s">
+      <c r="A73" s="25" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" t="s">
+      <c r="A74" s="25" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="75" spans="1:1">
-      <c r="A75" t="s">
+      <c r="A75" s="25" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="76" spans="1:1">
-      <c r="A76" t="s">
+      <c r="A76" s="25" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="77" spans="1:1">
-      <c r="A77" t="s">
+      <c r="A77" s="25" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="78" spans="1:1">
-      <c r="A78" t="s">
+      <c r="A78" s="25" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="79" spans="1:1">
-      <c r="A79" t="s">
+      <c r="A79" s="25" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="80" spans="1:1">
-      <c r="A80" t="s">
+      <c r="A80" s="25" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="81" spans="1:1">
-      <c r="A81" t="s">
+      <c r="A81" s="25" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="82" spans="1:1">
-      <c r="A82" t="s">
+      <c r="A82" s="25" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="83" spans="1:1">
-      <c r="A83" t="s">
+      <c r="A83" s="25" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="84" spans="1:1">
-      <c r="A84" t="s">
+      <c r="A84" s="25" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="85" spans="1:1">
-      <c r="A85" t="s">
+      <c r="A85" s="25" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="86" spans="1:1">
-      <c r="A86" t="s">
+      <c r="A86" s="25" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="87" spans="1:1">
-      <c r="A87" t="s">
+      <c r="A87" s="25" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="88" spans="1:1">
-      <c r="A88" t="s">
+      <c r="A88" s="25" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="89" spans="1:1">
-      <c r="A89" t="s">
+      <c r="A89" s="25" t="s">
         <v>383</v>
       </c>
     </row>
     <row r="90" spans="1:1">
-      <c r="A90" t="s">
+      <c r="A90" s="25" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="91" spans="1:1">
-      <c r="A91" t="s">
+      <c r="A91" s="25" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="92" spans="1:1">
-      <c r="A92" t="s">
+      <c r="A92" s="25" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="93" spans="1:1">
-      <c r="A93" t="s">
+      <c r="A93" s="25" t="s">
         <v>387</v>
       </c>
     </row>
     <row r="94" spans="1:1">
-      <c r="A94" t="s">
+      <c r="A94" s="25" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="95" spans="1:1">
-      <c r="A95" t="s">
+      <c r="A95" s="25" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="96" spans="1:1">
-      <c r="A96" t="s">
+      <c r="A96" s="25" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="97" spans="1:1">
-      <c r="A97" t="s">
+      <c r="A97" s="25" t="s">
         <v>391</v>
       </c>
     </row>
     <row r="98" spans="1:1">
-      <c r="A98" t="s">
+      <c r="A98" s="25" t="s">
         <v>392</v>
       </c>
     </row>
     <row r="99" spans="1:1">
-      <c r="A99" t="s">
+      <c r="A99" s="25" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="100" spans="1:1">
-      <c r="A100" t="s">
+      <c r="A100" s="25" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="101" spans="1:1">
-      <c r="A101" t="s">
+      <c r="A101" s="25" t="s">
         <v>395</v>
       </c>
     </row>
     <row r="102" spans="1:1">
-      <c r="A102" t="s">
+      <c r="A102" s="25" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="103" spans="1:1">
-      <c r="A103" t="s">
+      <c r="A103" s="25" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="104" spans="1:1">
-      <c r="A104" t="s">
+      <c r="A104" s="25" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="105" spans="1:1">
-      <c r="A105" t="s">
+      <c r="A105" s="25" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="106" spans="1:1">
-      <c r="A106" t="s">
+      <c r="A106" s="25" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="107" spans="1:1">
-      <c r="A107" t="s">
+      <c r="A107" s="25" t="s">
         <v>401</v>
       </c>
     </row>
     <row r="108" spans="1:1">
-      <c r="A108" t="s">
+      <c r="A108" s="25" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="109" spans="1:1">
-      <c r="A109" t="s">
+      <c r="A109" s="25" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="110" spans="1:1">
-      <c r="A110" t="s">
+      <c r="A110" s="25" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="111" spans="1:1">
-      <c r="A111" t="s">
+      <c r="A111" s="25" t="s">
         <v>405</v>
       </c>
     </row>
     <row r="112" spans="1:1">
-      <c r="A112" t="s">
+      <c r="A112" s="25" t="s">
         <v>406</v>
       </c>
     </row>
     <row r="113" spans="1:1">
-      <c r="A113" t="s">
+      <c r="A113" s="25" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="114" spans="1:1">
-      <c r="A114" t="s">
+      <c r="A114" s="25" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="115" spans="1:1">
-      <c r="A115" t="s">
+      <c r="A115" s="25" t="s">
         <v>409</v>
       </c>
     </row>
     <row r="116" spans="1:1">
-      <c r="A116" t="s">
+      <c r="A116" s="25" t="s">
         <v>410</v>
       </c>
     </row>
     <row r="117" spans="1:1">
-      <c r="A117" t="s">
+      <c r="A117" s="25" t="s">
         <v>411</v>
       </c>
     </row>
     <row r="118" spans="1:1">
-      <c r="A118" t="s">
+      <c r="A118" s="25" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="119" spans="1:1">
-      <c r="A119" t="s">
+      <c r="A119" s="25" t="s">
         <v>413</v>
       </c>
     </row>
     <row r="120" spans="1:1">
-      <c r="A120" t="s">
+      <c r="A120" s="25" t="s">
         <v>414</v>
       </c>
     </row>
     <row r="121" spans="1:1">
-      <c r="A121" t="s">
+      <c r="A121" s="25" t="s">
         <v>415</v>
       </c>
     </row>
     <row r="122" spans="1:1">
-      <c r="A122" t="s">
+      <c r="A122" s="25" t="s">
         <v>416</v>
       </c>
     </row>
     <row r="123" spans="1:1">
-      <c r="A123" t="s">
+      <c r="A123" s="25" t="s">
         <v>417</v>
       </c>
     </row>
     <row r="124" spans="1:1">
-      <c r="A124" t="s">
+      <c r="A124" s="25" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="125" spans="1:1">
-      <c r="A125" t="s">
+      <c r="A125" s="25" t="s">
         <v>419</v>
       </c>
     </row>
     <row r="126" spans="1:1">
-      <c r="A126" t="s">
+      <c r="A126" s="25" t="s">
         <v>420</v>
       </c>
     </row>
     <row r="127" spans="1:1">
-      <c r="A127" t="s">
+      <c r="A127" s="25" t="s">
         <v>421</v>
       </c>
     </row>
     <row r="128" spans="1:1">
-      <c r="A128" t="s">
+      <c r="A128" s="25" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="129" spans="1:1">
-      <c r="A129" t="s">
+      <c r="A129" s="25" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="130" spans="1:1">
-      <c r="A130" t="s">
+      <c r="A130" s="25" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="131" spans="1:1">
-      <c r="A131" t="s">
+      <c r="A131" s="25" t="s">
         <v>425</v>
       </c>
     </row>
     <row r="132" spans="1:1">
-      <c r="A132" t="s">
+      <c r="A132" s="25" t="s">
         <v>426</v>
       </c>
     </row>
     <row r="133" spans="1:1">
-      <c r="A133" t="s">
+      <c r="A133" s="25" t="s">
         <v>427</v>
       </c>
     </row>
     <row r="134" spans="1:1">
-      <c r="A134" t="s">
+      <c r="A134" s="25" t="s">
         <v>428</v>
       </c>
     </row>
     <row r="135" spans="1:1">
-      <c r="A135" t="s">
+      <c r="A135" s="25" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="136" spans="1:1">
-      <c r="A136" t="s">
+      <c r="A136" s="25" t="s">
         <v>430</v>
       </c>
     </row>
     <row r="137" spans="1:1">
-      <c r="A137" t="s">
+      <c r="A137" s="25" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="138" spans="1:1">
-      <c r="A138" t="s">
+      <c r="A138" s="25" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="139" spans="1:1">
-      <c r="A139" t="s">
+      <c r="A139" s="25" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="140" spans="1:1">
-      <c r="A140" t="s">
+      <c r="A140" s="25" t="s">
         <v>434</v>
       </c>
     </row>
     <row r="141" spans="1:1">
-      <c r="A141" t="s">
+      <c r="A141" s="25" t="s">
         <v>435</v>
       </c>
     </row>
     <row r="142" spans="1:1">
-      <c r="A142" t="s">
+      <c r="A142" s="25" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="143" spans="1:1">
-      <c r="A143" t="s">
+      <c r="A143" s="25" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="144" spans="1:1">
-      <c r="A144" t="s">
+      <c r="A144" s="25" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="145" spans="1:1">
-      <c r="A145" t="s">
+      <c r="A145" s="25" t="s">
         <v>439</v>
       </c>
     </row>
     <row r="146" spans="1:1">
-      <c r="A146" t="s">
+      <c r="A146" s="25" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="147" spans="1:1">
-      <c r="A147" t="s">
+      <c r="A147" s="25" t="s">
         <v>441</v>
       </c>
     </row>
     <row r="148" spans="1:1">
-      <c r="A148" t="s">
+      <c r="A148" s="25" t="s">
         <v>442</v>
       </c>
     </row>
     <row r="149" spans="1:1">
-      <c r="A149" t="s">
+      <c r="A149" s="25" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="150" spans="1:1">
-      <c r="A150" t="s">
+      <c r="A150" s="25" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="151" spans="1:1">
-      <c r="A151" t="s">
+      <c r="A151" s="25" t="s">
         <v>445</v>
       </c>
     </row>
     <row r="152" spans="1:1">
-      <c r="A152" t="s">
+      <c r="A152" s="25" t="s">
         <v>446</v>
       </c>
     </row>
     <row r="153" spans="1:1">
-      <c r="A153" t="s">
+      <c r="A153" s="25" t="s">
         <v>447</v>
       </c>
     </row>

</xml_diff>

<commit_message>
claude improving it further
</commit_message>
<xml_diff>
--- a/src/v2/tests/header_test.xlsx
+++ b/src/v2/tests/header_test.xlsx
@@ -1387,13 +1387,13 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1419,6 +1419,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFCC00"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1426,12 +1432,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1445,26 +1445,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color auto="1"/>
       </left>
@@ -1498,6 +1478,91 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="dotted">
         <color auto="1"/>
       </left>
@@ -1535,43 +1600,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color auto="1"/>
       </left>
@@ -1589,6 +1617,51 @@
       </right>
       <top/>
       <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -1603,83 +1676,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color auto="1"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
         <color auto="1"/>
       </right>
       <top style="thin">
@@ -1699,83 +1699,83 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2100,37 +2100,37 @@
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
-      <c r="J1" s="25">
+      <c r="J1" s="33">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,60,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="3"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="17"/>
     </row>
     <row r="2" spans="2:22">
-      <c r="B2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="7">
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="5">
         <f>IF($E$2="","Chose your language",VLOOKUP($E$2,Sprachversionen!$B:$BN,27,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="3">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,61,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
     </row>
     <row r="3" spans="2:22">
       <c r="B3" s="1">
@@ -2138,125 +2138,125 @@
         <v>0</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" s="7">
+      <c r="D3" s="5">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E3" s="23">
+      <c r="E3" s="30">
         <f>IF($E$2="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>0</v>
       </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
     </row>
     <row r="4" spans="2:22" ht="12" customHeight="1">
-      <c r="J4" s="6">
+      <c r="J4" s="4">
         <f>HYPERLINK(VLOOKUP($E$2,Sprachversionen!$B:$BN,62,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
     </row>
     <row r="5" spans="2:22">
-      <c r="B5" s="7">
+      <c r="B5" s="5">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,4,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="8"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="18"/>
     </row>
     <row r="6" spans="2:22">
-      <c r="B6" s="7">
+      <c r="B6" s="5">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,26,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" spans="2:22">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="J7" s="11"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="J7" s="19"/>
     </row>
     <row r="8" spans="2:22">
-      <c r="B8" s="7">
+      <c r="B8" s="5">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,5,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="26">
+      <c r="C8" s="5"/>
+      <c r="D8" s="34">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E8" s="10"/>
-      <c r="F8" s="26">
+      <c r="E8" s="7"/>
+      <c r="F8" s="34">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="J8" s="12"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="J8" s="20"/>
       <c r="K8">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,59,FALSE))</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:22">
-      <c r="B9" s="7">
+      <c r="B9" s="5">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,6,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="26">
+      <c r="C9" s="5"/>
+      <c r="D9" s="34">
         <f>D8</f>
         <v>0</v>
       </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="26">
+      <c r="E9" s="7"/>
+      <c r="F9" s="34">
         <f>F8</f>
         <v>0</v>
       </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="J9" s="13"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="J9" s="21"/>
     </row>
     <row r="10" spans="2:22" ht="13.5" customHeight="1"/>
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
-      <c r="B11" s="14"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16">
+      <c r="B11" s="22"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="8">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="9">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,12,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="8">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,13,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="8">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,14,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="10">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,15,FALSE))</f>
         <v>0</v>
       </c>
@@ -2272,173 +2272,172 @@
       <c r="R11" s="1"/>
     </row>
     <row r="12" spans="2:22">
-      <c r="B12" s="19">
+      <c r="B12" s="11">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,9,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="18"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" spans="2:22">
-      <c r="B13" s="20">
+      <c r="B13" s="12">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,10,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="18"/>
-      <c r="L13" s="24">
+      <c r="C13" s="12"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="10"/>
+      <c r="L13" s="31">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="M13" s="24" t="s">
+      <c r="M13" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="N13" s="24">
+      <c r="N13" s="31">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>0</v>
       </c>
-      <c r="O13" s="24">
+      <c r="O13" s="31">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="S13" s="24">
+      <c r="S13" s="31">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="T13" s="24" t="s">
+      <c r="T13" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="U13" s="24">
+      <c r="U13" s="31">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>0</v>
       </c>
-      <c r="V13" s="24">
+      <c r="V13" s="31">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:22">
-      <c r="B14" s="21"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="18"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="2:22">
-      <c r="B15" s="27">
+      <c r="B15" s="13">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,16,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C15" s="27"/>
-      <c r="D15" s="28">
-        <v>0</v>
-      </c>
-      <c r="E15" s="29"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="32"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="32">
+        <v>0</v>
+      </c>
+      <c r="E15" s="26"/>
+      <c r="F15" s="27"/>
+      <c r="H15" s="28"/>
     </row>
     <row r="16" spans="2:22">
-      <c r="B16" s="33">
+      <c r="B16" s="14">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,17,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C16" s="33"/>
-      <c r="D16" s="28">
-        <v>0</v>
-      </c>
-      <c r="E16" s="29"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="31">
+      <c r="C16" s="14"/>
+      <c r="D16" s="32">
+        <v>0</v>
+      </c>
+      <c r="E16" s="26"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="35">
         <f>IFERROR(F16/D16,0)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="32"/>
+      <c r="H16" s="28"/>
     </row>
     <row r="17" spans="2:8">
-      <c r="B17" s="33">
+      <c r="B17" s="14">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,18,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C17" s="33"/>
-      <c r="D17" s="28">
-        <v>0</v>
-      </c>
-      <c r="E17" s="29"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="31">
+      <c r="C17" s="14"/>
+      <c r="D17" s="32">
+        <v>0</v>
+      </c>
+      <c r="E17" s="26"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="35">
         <f>IFERROR(F17/D17,0)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="32"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="2:8">
-      <c r="B18" s="33">
+      <c r="B18" s="14">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C18" s="33"/>
-      <c r="D18" s="28">
-        <v>0</v>
-      </c>
-      <c r="E18" s="29"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="31">
+      <c r="C18" s="14"/>
+      <c r="D18" s="32">
+        <v>0</v>
+      </c>
+      <c r="E18" s="26"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="35">
         <f>IFERROR(F18/D18,0)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="32"/>
+      <c r="H18" s="28"/>
     </row>
     <row r="19" spans="2:8">
-      <c r="B19" s="33">
+      <c r="B19" s="14">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,20,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C19" s="33"/>
-      <c r="D19" s="28">
-        <v>0</v>
-      </c>
-      <c r="E19" s="29"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="31">
+      <c r="C19" s="14"/>
+      <c r="D19" s="32">
+        <v>0</v>
+      </c>
+      <c r="E19" s="26"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="35">
         <f>IFERROR(F19/D19,0)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="32"/>
+      <c r="H19" s="28"/>
     </row>
     <row r="20" spans="2:8">
-      <c r="B20" s="34">
+      <c r="B20" s="15">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,21,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C20" s="34"/>
-      <c r="D20" s="35">
+      <c r="C20" s="15"/>
+      <c r="D20" s="36">
         <f>SUMPRODUCT(ROUND(D15:D19, 2))</f>
         <v>0</v>
       </c>
-      <c r="E20" s="35">
+      <c r="E20" s="36">
         <f>SUMPRODUCT(ROUND(E15:E19, 2))</f>
         <v>0</v>
       </c>
-      <c r="F20" s="35">
+      <c r="F20" s="36">
         <f>SUMPRODUCT(ROUND(F15:F19, 2))</f>
         <v>0</v>
       </c>
-      <c r="G20" s="36">
+      <c r="G20" s="37">
         <f>IFERROR(INDEX($F$1:$F$1001,ROW())/INDEX($D$1:$D$1001,ROW()),0)</f>
         <v>0</v>
       </c>
-      <c r="H20" s="37"/>
+      <c r="H20" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="27">

</xml_diff>

<commit_message>
Improving speed and now working!
</commit_message>
<xml_diff>
--- a/src/v2/tests/header_test.xlsx
+++ b/src/v2/tests/header_test.xlsx
@@ -1379,6 +1379,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
@@ -1388,12 +1394,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1694,174 +1694,177 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2156,381 +2159,379 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:ALL20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" customWidth="1"/>
-    <col min="3" max="3" width="56.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" customWidth="1"/>
-    <col min="9" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" customWidth="1"/>
-    <col min="13" max="15" width="15.7109375" customWidth="1"/>
-    <col min="16" max="16" width="5.7109375" customWidth="1"/>
-    <col min="17" max="17" width="4.7109375" customWidth="1"/>
-    <col min="18" max="18" width="19.85546875" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" customWidth="1"/>
-    <col min="20" max="22" width="15.7109375" customWidth="1"/>
-    <col min="23" max="23" width="4.7109375" customWidth="1"/>
-    <col min="24" max="24" width="37.42578125" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="56.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="1" customWidth="1"/>
+    <col min="5" max="6" width="18.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="10" width="4.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" style="1" customWidth="1"/>
+    <col min="13" max="15" width="15.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="5.7109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="19.85546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" style="1" customWidth="1"/>
+    <col min="20" max="22" width="15.7109375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="4.7109375" style="1" customWidth="1"/>
+    <col min="24" max="24" width="37.42578125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5703125" style="1" customWidth="1"/>
+    <col min="26" max="1000" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:22">
-      <c r="B1" s="33">
+      <c r="B1" s="34">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,2,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="J1" s="34">
+      <c r="C1" s="2"/>
+      <c r="J1" s="35">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,60,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="18"/>
     </row>
     <row r="2" spans="2:22">
-      <c r="B2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="35">
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="36">
         <f>IF($E$2="","Chose your language",VLOOKUP($E$2,Sprachversionen!$B:$BN,27,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="36">
+      <c r="J2" s="37">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,61,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="2:22">
-      <c r="B3" s="33">
+      <c r="B3" s="34">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,3,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="35">
+      <c r="C3" s="2"/>
+      <c r="D3" s="36">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E3" s="37">
+      <c r="E3" s="38">
         <f>IF($E$2="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>0</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
     <row r="4" spans="2:22" ht="12" customHeight="1">
-      <c r="J4" s="38">
+      <c r="J4" s="39">
         <f>HYPERLINK(VLOOKUP($E$2,Sprachversionen!$B:$BN,62,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
     </row>
     <row r="5" spans="2:22">
-      <c r="B5" s="35">
+      <c r="B5" s="36">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,4,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="18"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="19"/>
     </row>
     <row r="6" spans="2:22">
-      <c r="B6" s="35">
+      <c r="B6" s="36">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,26,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
     </row>
     <row r="7" spans="2:22">
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="J7" s="19"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="J7" s="20"/>
     </row>
     <row r="8" spans="2:22">
-      <c r="B8" s="35">
+      <c r="B8" s="36">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,5,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="39">
+      <c r="C8" s="6"/>
+      <c r="D8" s="40">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="39">
+      <c r="E8" s="8"/>
+      <c r="F8" s="40">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="J8" s="20"/>
-      <c r="K8">
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="1">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,59,FALSE))</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:22">
-      <c r="B9" s="35">
+      <c r="B9" s="36">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,6,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="39">
+      <c r="C9" s="6"/>
+      <c r="D9" s="40">
         <f>D8</f>
         <v>0</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="39">
+      <c r="E9" s="8"/>
+      <c r="F9" s="40">
         <f>F8</f>
         <v>0</v>
       </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="J9" s="21"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="J9" s="22"/>
     </row>
     <row r="10" spans="2:22" ht="13.5" customHeight="1"/>
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
-      <c r="B11" s="22"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="40">
+      <c r="B11" s="23"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="41">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E11" s="41">
+      <c r="E11" s="42">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,12,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="F11" s="40">
+      <c r="F11" s="41">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,13,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="G11" s="40">
+      <c r="G11" s="41">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,14,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="H11" s="42">
+      <c r="H11" s="43">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,15,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="J11" s="33">
+      <c r="J11" s="34">
         <f>B18</f>
         <v>0</v>
       </c>
-      <c r="K11" s="1"/>
-      <c r="Q11" s="33">
+      <c r="K11" s="2"/>
+      <c r="Q11" s="34">
         <f>B18</f>
         <v>0</v>
       </c>
-      <c r="R11" s="1"/>
+      <c r="R11" s="2"/>
     </row>
     <row r="12" spans="2:22">
-      <c r="B12" s="43">
+      <c r="B12" s="44">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,9,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="10"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="11"/>
     </row>
     <row r="13" spans="2:22">
-      <c r="B13" s="44">
+      <c r="B13" s="45">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,10,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="10"/>
-      <c r="L13" s="45">
+      <c r="C13" s="13"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="11"/>
+      <c r="L13" s="46">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="M13" s="31" t="s">
+      <c r="M13" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="N13" s="45">
+      <c r="N13" s="46">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>0</v>
       </c>
-      <c r="O13" s="45">
+      <c r="O13" s="46">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="S13" s="45">
+      <c r="S13" s="46">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="T13" s="31" t="s">
+      <c r="T13" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="U13" s="45">
+      <c r="U13" s="46">
         <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
         <v>0</v>
       </c>
-      <c r="V13" s="45">
+      <c r="V13" s="46">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE))</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:22">
-      <c r="B14" s="24"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="10"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="11"/>
     </row>
     <row r="15" spans="2:22">
-      <c r="B15" s="46">
+      <c r="B15" s="47">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,16,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="32">
-        <v>0</v>
-      </c>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="28"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="33">
+        <v>0</v>
+      </c>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="29"/>
     </row>
     <row r="16" spans="2:22">
-      <c r="B16" s="47">
+      <c r="B16" s="48">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,17,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="32">
-        <v>0</v>
-      </c>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="48">
+      <c r="C16" s="15"/>
+      <c r="D16" s="33">
+        <v>0</v>
+      </c>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="49">
         <f>IFERROR(F16/D16,0)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="28"/>
+      <c r="H16" s="29"/>
     </row>
     <row r="17" spans="2:8">
-      <c r="B17" s="47">
+      <c r="B17" s="48">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,18,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="32">
-        <v>0</v>
-      </c>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="48">
+      <c r="C17" s="15"/>
+      <c r="D17" s="33">
+        <v>0</v>
+      </c>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="49">
         <f>IFERROR(F17/D17,0)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="28"/>
+      <c r="H17" s="29"/>
     </row>
     <row r="18" spans="2:8">
-      <c r="B18" s="47">
+      <c r="B18" s="48">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="32">
-        <v>0</v>
-      </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="48">
+      <c r="C18" s="15"/>
+      <c r="D18" s="33">
+        <v>0</v>
+      </c>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="49">
         <f>IFERROR(F18/D18,0)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="28"/>
+      <c r="H18" s="29"/>
     </row>
     <row r="19" spans="2:8">
-      <c r="B19" s="47">
+      <c r="B19" s="48">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,20,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="32">
-        <v>0</v>
-      </c>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="48">
+      <c r="C19" s="15"/>
+      <c r="D19" s="33">
+        <v>0</v>
+      </c>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="49">
         <f>IFERROR(F19/D19,0)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="28"/>
+      <c r="H19" s="29"/>
     </row>
     <row r="20" spans="2:8">
-      <c r="B20" s="49">
+      <c r="B20" s="50">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,21,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="50">
+      <c r="C20" s="16"/>
+      <c r="D20" s="51">
         <f>SUMPRODUCT(ROUND(D15:D19, 2))</f>
         <v>0</v>
       </c>
-      <c r="E20" s="50">
+      <c r="E20" s="51">
         <f>SUMPRODUCT(ROUND(E15:E19, 2))</f>
         <v>0</v>
       </c>
-      <c r="F20" s="50">
+      <c r="F20" s="51">
         <f>SUMPRODUCT(ROUND(F15:F19, 2))</f>
         <v>0</v>
       </c>
-      <c r="G20" s="51">
+      <c r="G20" s="52">
         <f>IFERROR(INDEX($F$1:$F$1001,ROW())/INDEX($D$1:$D$1001,ROW()),0)</f>
         <v>0</v>
       </c>
-      <c r="H20" s="29"/>
+      <c r="H20" s="30"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <protectedRanges>
-    <protectedRange sqref="A1:NTP10000" name="Range1"/>
-  </protectedRanges>
   <mergeCells count="27">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -2575,1697 +2576,1697 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:63">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="C1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="52" t="s">
+      <c r="E1" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="52" t="s">
+      <c r="F1" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="52" t="s">
+      <c r="G1" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="52" t="s">
+      <c r="H1" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="52" t="s">
+      <c r="I1" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="52" t="s">
+      <c r="J1" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="52" t="s">
+      <c r="K1" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="52" t="s">
+      <c r="L1" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="52" t="s">
+      <c r="M1" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="52" t="s">
+      <c r="N1" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="52" t="s">
+      <c r="O1" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="P1" s="52" t="s">
+      <c r="P1" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" s="52" t="s">
+      <c r="Q1" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="R1" s="52" t="s">
+      <c r="R1" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="S1" s="52" t="s">
+      <c r="S1" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="T1" s="52" t="s">
+      <c r="T1" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="U1" s="52" t="s">
+      <c r="U1" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="V1" s="52" t="s">
+      <c r="V1" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="W1" s="52" t="s">
+      <c r="W1" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="X1" s="52" t="s">
+      <c r="X1" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="Y1" s="52" t="s">
+      <c r="Y1" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="Z1" s="52" t="s">
+      <c r="Z1" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="AA1" s="52" t="s">
+      <c r="AA1" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="AB1" s="52" t="s">
+      <c r="AB1" s="53" t="s">
         <v>29</v>
       </c>
-      <c r="AC1" s="52" t="s">
+      <c r="AC1" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="AD1" s="52" t="s">
+      <c r="AD1" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="AE1" s="52" t="s">
+      <c r="AE1" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="AF1" s="52" t="s">
+      <c r="AF1" s="53" t="s">
         <v>33</v>
       </c>
-      <c r="AG1" s="52" t="s">
+      <c r="AG1" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="AH1" s="52" t="s">
+      <c r="AH1" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="AI1" s="52" t="s">
+      <c r="AI1" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="AJ1" s="52" t="s">
+      <c r="AJ1" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="AK1" s="52" t="s">
+      <c r="AK1" s="53" t="s">
         <v>38</v>
       </c>
-      <c r="AL1" s="52" t="s">
+      <c r="AL1" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="AM1" s="52" t="s">
+      <c r="AM1" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="AN1" s="52" t="s">
+      <c r="AN1" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="AO1" s="52" t="s">
+      <c r="AO1" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="AP1" s="52" t="s">
+      <c r="AP1" s="53" t="s">
         <v>43</v>
       </c>
-      <c r="AQ1" s="52" t="s">
+      <c r="AQ1" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="AR1" s="52" t="s">
+      <c r="AR1" s="53" t="s">
         <v>45</v>
       </c>
-      <c r="AS1" s="52" t="s">
+      <c r="AS1" s="53" t="s">
         <v>46</v>
       </c>
-      <c r="AT1" s="52" t="s">
+      <c r="AT1" s="53" t="s">
         <v>47</v>
       </c>
-      <c r="AU1" s="52" t="s">
+      <c r="AU1" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="AV1" s="52" t="s">
+      <c r="AV1" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="AW1" s="52" t="s">
+      <c r="AW1" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="AX1" s="52" t="s">
+      <c r="AX1" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="AY1" s="52" t="s">
+      <c r="AY1" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="AZ1" s="52" t="s">
+      <c r="AZ1" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="BA1" s="52" t="s">
+      <c r="BA1" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="BB1" s="52" t="s">
+      <c r="BB1" s="53" t="s">
         <v>55</v>
       </c>
-      <c r="BC1" s="52" t="s">
+      <c r="BC1" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="BD1" s="52" t="s">
+      <c r="BD1" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="BE1" s="52" t="s">
+      <c r="BE1" s="53" t="s">
         <v>58</v>
       </c>
-      <c r="BF1" s="52" t="s">
+      <c r="BF1" s="53" t="s">
         <v>59</v>
       </c>
-      <c r="BG1" s="52" t="s">
+      <c r="BG1" s="53" t="s">
         <v>60</v>
       </c>
-      <c r="BH1" s="52" t="s">
+      <c r="BH1" s="53" t="s">
         <v>61</v>
       </c>
-      <c r="BI1" s="52" t="s">
+      <c r="BI1" s="53" t="s">
         <v>62</v>
       </c>
-      <c r="BJ1" s="52" t="s">
+      <c r="BJ1" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="BK1" s="52" t="s">
+      <c r="BK1" s="53" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:63">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="53" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="53" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="52" t="s">
+      <c r="D2" s="53" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="52" t="s">
+      <c r="E2" s="53" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="53" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="52" t="s">
+      <c r="G2" s="53" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="52" t="s">
+      <c r="H2" s="53" t="s">
         <v>72</v>
       </c>
-      <c r="I2" s="52" t="s">
+      <c r="I2" s="53" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="52" t="s">
+      <c r="J2" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="K2" s="52" t="s">
+      <c r="K2" s="53" t="s">
         <v>75</v>
       </c>
-      <c r="L2" s="52" t="s">
+      <c r="L2" s="53" t="s">
         <v>76</v>
       </c>
-      <c r="M2" s="52" t="s">
+      <c r="M2" s="53" t="s">
         <v>77</v>
       </c>
-      <c r="N2" s="52" t="s">
+      <c r="N2" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="O2" s="52" t="s">
+      <c r="O2" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="P2" s="52" t="s">
+      <c r="P2" s="53" t="s">
         <v>80</v>
       </c>
-      <c r="Q2" s="52" t="s">
+      <c r="Q2" s="53" t="s">
         <v>81</v>
       </c>
-      <c r="R2" s="52" t="s">
+      <c r="R2" s="53" t="s">
         <v>82</v>
       </c>
-      <c r="S2" s="52" t="s">
+      <c r="S2" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="T2" s="52" t="s">
+      <c r="T2" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="U2" s="52" t="s">
+      <c r="U2" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="V2" s="52" t="s">
+      <c r="V2" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="W2" s="52" t="s">
+      <c r="W2" s="53" t="s">
         <v>87</v>
       </c>
-      <c r="X2" s="52" t="s">
+      <c r="X2" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="Y2" s="52" t="s">
+      <c r="Y2" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="Z2" s="52" t="s">
+      <c r="Z2" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="AA2" s="52" t="s">
+      <c r="AA2" s="53" t="s">
         <v>91</v>
       </c>
-      <c r="AB2" s="52" t="s">
+      <c r="AB2" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="AC2" s="52" t="s">
+      <c r="AC2" s="53" t="s">
         <v>93</v>
       </c>
-      <c r="AD2" s="52" t="s">
+      <c r="AD2" s="53" t="s">
         <v>94</v>
       </c>
-      <c r="AE2" s="52" t="s">
+      <c r="AE2" s="53" t="s">
         <v>95</v>
       </c>
-      <c r="AF2" s="52" t="s">
+      <c r="AF2" s="53" t="s">
         <v>96</v>
       </c>
-      <c r="AG2" s="52" t="s">
+      <c r="AG2" s="53" t="s">
         <v>97</v>
       </c>
-      <c r="AH2" s="52" t="s">
+      <c r="AH2" s="53" t="s">
         <v>98</v>
       </c>
-      <c r="AI2" s="52" t="s">
+      <c r="AI2" s="53" t="s">
         <v>99</v>
       </c>
-      <c r="AJ2" s="52" t="s">
+      <c r="AJ2" s="53" t="s">
         <v>100</v>
       </c>
-      <c r="AK2" s="52" t="s">
+      <c r="AK2" s="53" t="s">
         <v>101</v>
       </c>
-      <c r="AL2" s="52" t="s">
+      <c r="AL2" s="53" t="s">
         <v>102</v>
       </c>
-      <c r="AM2" s="52" t="s">
+      <c r="AM2" s="53" t="s">
         <v>103</v>
       </c>
-      <c r="AN2" s="52" t="s">
+      <c r="AN2" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="AO2" s="52" t="s">
+      <c r="AO2" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="AP2" s="52" t="s">
+      <c r="AP2" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="AQ2" s="52" t="s">
+      <c r="AQ2" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="AR2" s="52" t="s">
+      <c r="AR2" s="53" t="s">
         <v>106</v>
       </c>
-      <c r="AS2" s="52" t="s">
+      <c r="AS2" s="53" t="s">
         <v>107</v>
       </c>
-      <c r="AT2" s="52" t="s">
+      <c r="AT2" s="53" t="s">
         <v>108</v>
       </c>
-      <c r="AU2" s="52" t="s">
+      <c r="AU2" s="53" t="s">
         <v>109</v>
       </c>
-      <c r="AV2" s="52" t="s">
+      <c r="AV2" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="AW2" s="52" t="s">
+      <c r="AW2" s="53" t="s">
         <v>110</v>
       </c>
-      <c r="AX2" s="52" t="s">
+      <c r="AX2" s="53" t="s">
         <v>111</v>
       </c>
-      <c r="AY2" s="52" t="s">
+      <c r="AY2" s="53" t="s">
         <v>112</v>
       </c>
-      <c r="AZ2" s="52" t="s">
+      <c r="AZ2" s="53" t="s">
         <v>113</v>
       </c>
-      <c r="BA2" s="52" t="s">
+      <c r="BA2" s="53" t="s">
         <v>114</v>
       </c>
-      <c r="BB2" s="52" t="s">
+      <c r="BB2" s="53" t="s">
         <v>115</v>
       </c>
-      <c r="BC2" s="52" t="s">
+      <c r="BC2" s="53" t="s">
         <v>116</v>
       </c>
-      <c r="BD2" s="52" t="s">
+      <c r="BD2" s="53" t="s">
         <v>117</v>
       </c>
-      <c r="BE2" s="52" t="s">
+      <c r="BE2" s="53" t="s">
         <v>118</v>
       </c>
-      <c r="BF2" s="52" t="s">
+      <c r="BF2" s="53" t="s">
         <v>119</v>
       </c>
-      <c r="BG2" s="52" t="s">
+      <c r="BG2" s="53" t="s">
         <v>120</v>
       </c>
-      <c r="BH2" s="52" t="s">
+      <c r="BH2" s="53" t="s">
         <v>121</v>
       </c>
-      <c r="BI2" s="52" t="s">
+      <c r="BI2" s="53" t="s">
         <v>122</v>
       </c>
-      <c r="BJ2" s="52" t="s">
+      <c r="BJ2" s="53" t="s">
         <v>123</v>
       </c>
-      <c r="BK2" s="52" t="s">
+      <c r="BK2" s="53" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:63">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="53" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="52" t="s">
+      <c r="B3" s="53" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="52" t="s">
+      <c r="C3" s="53" t="s">
         <v>127</v>
       </c>
-      <c r="D3" s="52" t="s">
+      <c r="D3" s="53" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="52" t="s">
+      <c r="E3" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="F3" s="52" t="s">
+      <c r="F3" s="53" t="s">
         <v>130</v>
       </c>
-      <c r="G3" s="52" t="s">
+      <c r="G3" s="53" t="s">
         <v>131</v>
       </c>
-      <c r="H3" s="52" t="s">
+      <c r="H3" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="I3" s="52" t="s">
+      <c r="I3" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="J3" s="52" t="s">
+      <c r="J3" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="K3" s="52" t="s">
+      <c r="K3" s="53" t="s">
         <v>134</v>
       </c>
-      <c r="L3" s="52" t="s">
+      <c r="L3" s="53" t="s">
         <v>135</v>
       </c>
-      <c r="M3" s="52" t="s">
+      <c r="M3" s="53" t="s">
         <v>136</v>
       </c>
-      <c r="N3" s="52" t="s">
+      <c r="N3" s="53" t="s">
         <v>137</v>
       </c>
-      <c r="O3" s="52" t="s">
+      <c r="O3" s="53" t="s">
         <v>138</v>
       </c>
-      <c r="P3" s="52" t="s">
+      <c r="P3" s="53" t="s">
         <v>139</v>
       </c>
-      <c r="Q3" s="52" t="s">
+      <c r="Q3" s="53" t="s">
         <v>140</v>
       </c>
-      <c r="R3" s="52" t="s">
+      <c r="R3" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="S3" s="52" t="s">
+      <c r="S3" s="53" t="s">
         <v>142</v>
       </c>
-      <c r="T3" s="52" t="s">
+      <c r="T3" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="U3" s="52" t="s">
+      <c r="U3" s="53" t="s">
         <v>144</v>
       </c>
-      <c r="V3" s="52" t="s">
+      <c r="V3" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="W3" s="52" t="s">
+      <c r="W3" s="53" t="s">
         <v>87</v>
       </c>
-      <c r="X3" s="52" t="s">
+      <c r="X3" s="53" t="s">
         <v>146</v>
       </c>
-      <c r="Y3" s="52" t="s">
+      <c r="Y3" s="53" t="s">
         <v>147</v>
       </c>
-      <c r="Z3" s="52" t="s">
+      <c r="Z3" s="53" t="s">
         <v>148</v>
       </c>
-      <c r="AA3" s="52" t="s">
+      <c r="AA3" s="53" t="s">
         <v>149</v>
       </c>
-      <c r="AB3" s="52" t="s">
+      <c r="AB3" s="53" t="s">
         <v>150</v>
       </c>
-      <c r="AC3" s="52" t="s">
+      <c r="AC3" s="53" t="s">
         <v>151</v>
       </c>
-      <c r="AD3" s="52" t="s">
+      <c r="AD3" s="53" t="s">
         <v>152</v>
       </c>
-      <c r="AE3" s="52" t="s">
+      <c r="AE3" s="53" t="s">
         <v>153</v>
       </c>
-      <c r="AF3" s="52" t="s">
+      <c r="AF3" s="53" t="s">
         <v>154</v>
       </c>
-      <c r="AG3" s="52" t="s">
+      <c r="AG3" s="53" t="s">
         <v>155</v>
       </c>
-      <c r="AH3" s="52" t="s">
+      <c r="AH3" s="53" t="s">
         <v>156</v>
       </c>
-      <c r="AI3" s="52" t="s">
+      <c r="AI3" s="53" t="s">
         <v>157</v>
       </c>
-      <c r="AJ3" s="52" t="s">
+      <c r="AJ3" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="AK3" s="52" t="s">
+      <c r="AK3" s="53" t="s">
         <v>159</v>
       </c>
-      <c r="AL3" s="52" t="s">
+      <c r="AL3" s="53" t="s">
         <v>160</v>
       </c>
-      <c r="AM3" s="52" t="s">
+      <c r="AM3" s="53" t="s">
         <v>161</v>
       </c>
-      <c r="AN3" s="52" t="s">
+      <c r="AN3" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="AO3" s="52" t="s">
+      <c r="AO3" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="AP3" s="52" t="s">
+      <c r="AP3" s="53" t="s">
         <v>162</v>
       </c>
-      <c r="AQ3" s="52" t="s">
+      <c r="AQ3" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="AR3" s="52" t="s">
+      <c r="AR3" s="53" t="s">
         <v>163</v>
       </c>
-      <c r="AS3" s="52" t="s">
+      <c r="AS3" s="53" t="s">
         <v>164</v>
       </c>
-      <c r="AT3" s="52" t="s">
+      <c r="AT3" s="53" t="s">
         <v>165</v>
       </c>
-      <c r="AU3" s="52" t="s">
+      <c r="AU3" s="53" t="s">
         <v>166</v>
       </c>
-      <c r="AV3" s="52" t="s">
+      <c r="AV3" s="53" t="s">
         <v>167</v>
       </c>
-      <c r="AW3" s="52" t="s">
+      <c r="AW3" s="53" t="s">
         <v>168</v>
       </c>
-      <c r="AX3" s="52" t="s">
+      <c r="AX3" s="53" t="s">
         <v>169</v>
       </c>
-      <c r="AY3" s="52" t="s">
+      <c r="AY3" s="53" t="s">
         <v>170</v>
       </c>
-      <c r="AZ3" s="52" t="s">
+      <c r="AZ3" s="53" t="s">
         <v>171</v>
       </c>
-      <c r="BA3" s="52" t="s">
+      <c r="BA3" s="53" t="s">
         <v>172</v>
       </c>
-      <c r="BB3" s="52" t="s">
+      <c r="BB3" s="53" t="s">
         <v>173</v>
       </c>
-      <c r="BC3" s="52" t="s">
+      <c r="BC3" s="53" t="s">
         <v>174</v>
       </c>
-      <c r="BD3" s="52" t="s">
+      <c r="BD3" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="BE3" s="52" t="s">
+      <c r="BE3" s="53" t="s">
         <v>176</v>
       </c>
-      <c r="BF3" s="52" t="s">
+      <c r="BF3" s="53" t="s">
         <v>177</v>
       </c>
-      <c r="BG3" s="52" t="s">
+      <c r="BG3" s="53" t="s">
         <v>178</v>
       </c>
-      <c r="BH3" s="52" t="s">
+      <c r="BH3" s="53" t="s">
         <v>179</v>
       </c>
-      <c r="BI3" s="52" t="s">
+      <c r="BI3" s="53" t="s">
         <v>180</v>
       </c>
-      <c r="BJ3" s="52" t="s">
+      <c r="BJ3" s="53" t="s">
         <v>181</v>
       </c>
-      <c r="BK3" s="52" t="s">
+      <c r="BK3" s="53" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:63">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="53" t="s">
         <v>183</v>
       </c>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="53" t="s">
         <v>184</v>
       </c>
-      <c r="C4" s="52" t="s">
+      <c r="C4" s="53" t="s">
         <v>185</v>
       </c>
-      <c r="D4" s="52" t="s">
+      <c r="D4" s="53" t="s">
         <v>186</v>
       </c>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="53" t="s">
         <v>187</v>
       </c>
-      <c r="F4" s="52" t="s">
+      <c r="F4" s="53" t="s">
         <v>188</v>
       </c>
-      <c r="G4" s="52" t="s">
+      <c r="G4" s="53" t="s">
         <v>189</v>
       </c>
-      <c r="H4" s="52" t="s">
+      <c r="H4" s="53" t="s">
         <v>190</v>
       </c>
-      <c r="I4" s="52" t="s">
+      <c r="I4" s="53" t="s">
         <v>191</v>
       </c>
-      <c r="J4" s="52" t="s">
+      <c r="J4" s="53" t="s">
         <v>192</v>
       </c>
-      <c r="K4" s="52" t="s">
+      <c r="K4" s="53" t="s">
         <v>193</v>
       </c>
-      <c r="L4" s="52" t="s">
+      <c r="L4" s="53" t="s">
         <v>194</v>
       </c>
-      <c r="M4" s="52" t="s">
+      <c r="M4" s="53" t="s">
         <v>195</v>
       </c>
-      <c r="N4" s="52" t="s">
+      <c r="N4" s="53" t="s">
         <v>196</v>
       </c>
-      <c r="O4" s="52" t="s">
+      <c r="O4" s="53" t="s">
         <v>197</v>
       </c>
-      <c r="P4" s="52" t="s">
+      <c r="P4" s="53" t="s">
         <v>198</v>
       </c>
-      <c r="Q4" s="52" t="s">
+      <c r="Q4" s="53" t="s">
         <v>199</v>
       </c>
-      <c r="R4" s="52" t="s">
+      <c r="R4" s="53" t="s">
         <v>200</v>
       </c>
-      <c r="S4" s="52" t="s">
+      <c r="S4" s="53" t="s">
         <v>201</v>
       </c>
-      <c r="T4" s="52" t="s">
+      <c r="T4" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="U4" s="52" t="s">
+      <c r="U4" s="53" t="s">
         <v>203</v>
       </c>
-      <c r="V4" s="52" t="s">
+      <c r="V4" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="W4" s="52" t="s">
+      <c r="W4" s="53" t="s">
         <v>204</v>
       </c>
-      <c r="X4" s="52" t="s">
+      <c r="X4" s="53" t="s">
         <v>205</v>
       </c>
-      <c r="Y4" s="52" t="s">
+      <c r="Y4" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="Z4" s="52" t="s">
+      <c r="Z4" s="53" t="s">
         <v>207</v>
       </c>
-      <c r="AA4" s="52" t="s">
+      <c r="AA4" s="53" t="s">
         <v>208</v>
       </c>
-      <c r="AB4" s="52" t="s">
+      <c r="AB4" s="53" t="s">
         <v>209</v>
       </c>
-      <c r="AC4" s="52" t="s">
+      <c r="AC4" s="53" t="s">
         <v>210</v>
       </c>
-      <c r="AD4" s="52" t="s">
+      <c r="AD4" s="53" t="s">
         <v>211</v>
       </c>
-      <c r="AE4" s="52" t="s">
+      <c r="AE4" s="53" t="s">
         <v>212</v>
       </c>
-      <c r="AF4" s="52" t="s">
+      <c r="AF4" s="53" t="s">
         <v>213</v>
       </c>
-      <c r="AG4" s="52" t="s">
+      <c r="AG4" s="53" t="s">
         <v>214</v>
       </c>
-      <c r="AH4" s="52" t="s">
+      <c r="AH4" s="53" t="s">
         <v>215</v>
       </c>
-      <c r="AI4" s="52" t="s">
+      <c r="AI4" s="53" t="s">
         <v>216</v>
       </c>
-      <c r="AJ4" s="52" t="s">
+      <c r="AJ4" s="53" t="s">
         <v>217</v>
       </c>
-      <c r="AK4" s="52" t="s">
+      <c r="AK4" s="53" t="s">
         <v>218</v>
       </c>
-      <c r="AL4" s="52" t="s">
+      <c r="AL4" s="53" t="s">
         <v>219</v>
       </c>
-      <c r="AM4" s="52" t="s">
+      <c r="AM4" s="53" t="s">
         <v>220</v>
       </c>
-      <c r="AN4" s="52" t="s">
+      <c r="AN4" s="53" t="s">
         <v>221</v>
       </c>
-      <c r="AO4" s="52" t="s">
+      <c r="AO4" s="53" t="s">
         <v>222</v>
       </c>
-      <c r="AP4" s="52" t="s">
+      <c r="AP4" s="53" t="s">
         <v>223</v>
       </c>
-      <c r="AQ4" s="52" t="s">
+      <c r="AQ4" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="AR4" s="52" t="s">
+      <c r="AR4" s="53" t="s">
         <v>224</v>
       </c>
-      <c r="AS4" s="52" t="s">
+      <c r="AS4" s="53" t="s">
         <v>225</v>
       </c>
-      <c r="AT4" s="52" t="s">
+      <c r="AT4" s="53" t="s">
         <v>226</v>
       </c>
-      <c r="AU4" s="52" t="s">
+      <c r="AU4" s="53" t="s">
         <v>227</v>
       </c>
-      <c r="AV4" s="52" t="s">
+      <c r="AV4" s="53" t="s">
         <v>228</v>
       </c>
-      <c r="AW4" s="52" t="s">
+      <c r="AW4" s="53" t="s">
         <v>229</v>
       </c>
-      <c r="AX4" s="52" t="s">
+      <c r="AX4" s="53" t="s">
         <v>230</v>
       </c>
-      <c r="AY4" s="52" t="s">
+      <c r="AY4" s="53" t="s">
         <v>231</v>
       </c>
-      <c r="AZ4" s="52" t="s">
+      <c r="AZ4" s="53" t="s">
         <v>232</v>
       </c>
-      <c r="BA4" s="52" t="s">
+      <c r="BA4" s="53" t="s">
         <v>233</v>
       </c>
-      <c r="BB4" s="52" t="s">
+      <c r="BB4" s="53" t="s">
         <v>234</v>
       </c>
-      <c r="BC4" s="52" t="s">
+      <c r="BC4" s="53" t="s">
         <v>235</v>
       </c>
-      <c r="BD4" s="52" t="s">
+      <c r="BD4" s="53" t="s">
         <v>236</v>
       </c>
-      <c r="BE4" s="52" t="s">
+      <c r="BE4" s="53" t="s">
         <v>237</v>
       </c>
-      <c r="BF4" s="52" t="s">
+      <c r="BF4" s="53" t="s">
         <v>238</v>
       </c>
-      <c r="BG4" s="52" t="s">
+      <c r="BG4" s="53" t="s">
         <v>178</v>
       </c>
-      <c r="BH4" s="52" t="s">
+      <c r="BH4" s="53" t="s">
         <v>239</v>
       </c>
-      <c r="BI4" s="52" t="s">
+      <c r="BI4" s="53" t="s">
         <v>240</v>
       </c>
-      <c r="BJ4" s="52" t="s">
+      <c r="BJ4" s="53" t="s">
         <v>241</v>
       </c>
-      <c r="BK4" s="52" t="s">
+      <c r="BK4" s="53" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:63">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="53" t="s">
         <v>243</v>
       </c>
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="53" t="s">
         <v>244</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="53" t="s">
         <v>245</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="53" t="s">
         <v>246</v>
       </c>
-      <c r="E5" s="52" t="s">
+      <c r="E5" s="53" t="s">
         <v>247</v>
       </c>
-      <c r="F5" s="52" t="s">
+      <c r="F5" s="53" t="s">
         <v>248</v>
       </c>
-      <c r="G5" s="52" t="s">
+      <c r="G5" s="53" t="s">
         <v>249</v>
       </c>
-      <c r="H5" s="52" t="s">
+      <c r="H5" s="53" t="s">
         <v>190</v>
       </c>
-      <c r="I5" s="52" t="s">
+      <c r="I5" s="53" t="s">
         <v>250</v>
       </c>
-      <c r="J5" s="52" t="s">
+      <c r="J5" s="53" t="s">
         <v>251</v>
       </c>
-      <c r="K5" s="52" t="s">
+      <c r="K5" s="53" t="s">
         <v>252</v>
       </c>
-      <c r="L5" s="52" t="s">
+      <c r="L5" s="53" t="s">
         <v>253</v>
       </c>
-      <c r="M5" s="52" t="s">
+      <c r="M5" s="53" t="s">
         <v>254</v>
       </c>
-      <c r="N5" s="52" t="s">
+      <c r="N5" s="53" t="s">
         <v>255</v>
       </c>
-      <c r="O5" s="52" t="s">
+      <c r="O5" s="53" t="s">
         <v>256</v>
       </c>
-      <c r="P5" s="52" t="s">
+      <c r="P5" s="53" t="s">
         <v>257</v>
       </c>
-      <c r="Q5" s="52" t="s">
+      <c r="Q5" s="53" t="s">
         <v>258</v>
       </c>
-      <c r="R5" s="52" t="s">
+      <c r="R5" s="53" t="s">
         <v>259</v>
       </c>
-      <c r="S5" s="52" t="s">
+      <c r="S5" s="53" t="s">
         <v>260</v>
       </c>
-      <c r="T5" s="52" t="s">
+      <c r="T5" s="53" t="s">
         <v>261</v>
       </c>
-      <c r="U5" s="52" t="s">
+      <c r="U5" s="53" t="s">
         <v>262</v>
       </c>
-      <c r="V5" s="52" t="s">
+      <c r="V5" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="W5" s="52" t="s">
+      <c r="W5" s="53" t="s">
         <v>263</v>
       </c>
-      <c r="X5" s="52" t="s">
+      <c r="X5" s="53" t="s">
         <v>264</v>
       </c>
-      <c r="Y5" s="52" t="s">
+      <c r="Y5" s="53" t="s">
         <v>265</v>
       </c>
-      <c r="Z5" s="52" t="s">
+      <c r="Z5" s="53" t="s">
         <v>266</v>
       </c>
-      <c r="AA5" s="52" t="s">
+      <c r="AA5" s="53" t="s">
         <v>267</v>
       </c>
-      <c r="AB5" s="52" t="s">
+      <c r="AB5" s="53" t="s">
         <v>209</v>
       </c>
-      <c r="AC5" s="52" t="s">
+      <c r="AC5" s="53" t="s">
         <v>268</v>
       </c>
-      <c r="AD5" s="52" t="s">
+      <c r="AD5" s="53" t="s">
         <v>269</v>
       </c>
-      <c r="AE5" s="52" t="s">
+      <c r="AE5" s="53" t="s">
         <v>270</v>
       </c>
-      <c r="AF5" s="52" t="s">
+      <c r="AF5" s="53" t="s">
         <v>271</v>
       </c>
-      <c r="AG5" s="52" t="s">
+      <c r="AG5" s="53" t="s">
         <v>272</v>
       </c>
-      <c r="AH5" s="52" t="s">
+      <c r="AH5" s="53" t="s">
         <v>273</v>
       </c>
-      <c r="AI5" s="52" t="s">
+      <c r="AI5" s="53" t="s">
         <v>274</v>
       </c>
-      <c r="AJ5" s="52" t="s">
+      <c r="AJ5" s="53" t="s">
         <v>275</v>
       </c>
-      <c r="AK5" s="52" t="s">
+      <c r="AK5" s="53" t="s">
         <v>276</v>
       </c>
-      <c r="AL5" s="52" t="s">
+      <c r="AL5" s="53" t="s">
         <v>277</v>
       </c>
-      <c r="AM5" s="52" t="s">
+      <c r="AM5" s="53" t="s">
         <v>278</v>
       </c>
-      <c r="AN5" s="52" t="s">
+      <c r="AN5" s="53" t="s">
         <v>279</v>
       </c>
-      <c r="AO5" s="52" t="s">
+      <c r="AO5" s="53" t="s">
         <v>280</v>
       </c>
-      <c r="AP5" s="52" t="s">
+      <c r="AP5" s="53" t="s">
         <v>281</v>
       </c>
-      <c r="AQ5" s="52" t="s">
+      <c r="AQ5" s="53" t="s">
         <v>86</v>
       </c>
-      <c r="AR5" s="52" t="s">
+      <c r="AR5" s="53" t="s">
         <v>282</v>
       </c>
-      <c r="AS5" s="52" t="s">
+      <c r="AS5" s="53" t="s">
         <v>283</v>
       </c>
-      <c r="AT5" s="52" t="s">
+      <c r="AT5" s="53" t="s">
         <v>284</v>
       </c>
-      <c r="AU5" s="52" t="s">
+      <c r="AU5" s="53" t="s">
         <v>285</v>
       </c>
-      <c r="AV5" s="52" t="s">
+      <c r="AV5" s="53" t="s">
         <v>228</v>
       </c>
-      <c r="AW5" s="52" t="s">
+      <c r="AW5" s="53" t="s">
         <v>286</v>
       </c>
-      <c r="AX5" s="52" t="s">
+      <c r="AX5" s="53" t="s">
         <v>287</v>
       </c>
-      <c r="AY5" s="52" t="s">
+      <c r="AY5" s="53" t="s">
         <v>288</v>
       </c>
-      <c r="AZ5" s="52" t="s">
+      <c r="AZ5" s="53" t="s">
         <v>289</v>
       </c>
-      <c r="BA5" s="52" t="s">
+      <c r="BA5" s="53" t="s">
         <v>290</v>
       </c>
-      <c r="BB5" s="52" t="s">
+      <c r="BB5" s="53" t="s">
         <v>291</v>
       </c>
-      <c r="BC5" s="52" t="s">
+      <c r="BC5" s="53" t="s">
         <v>292</v>
       </c>
-      <c r="BD5" s="52" t="s">
+      <c r="BD5" s="53" t="s">
         <v>293</v>
       </c>
-      <c r="BE5" s="52" t="s">
+      <c r="BE5" s="53" t="s">
         <v>294</v>
       </c>
-      <c r="BF5" s="52" t="s">
+      <c r="BF5" s="53" t="s">
         <v>295</v>
       </c>
-      <c r="BG5" s="52" t="s">
+      <c r="BG5" s="53" t="s">
         <v>178</v>
       </c>
-      <c r="BH5" s="52" t="s">
+      <c r="BH5" s="53" t="s">
         <v>296</v>
       </c>
-      <c r="BI5" s="52" t="s">
+      <c r="BI5" s="53" t="s">
         <v>297</v>
       </c>
-      <c r="BJ5" s="52" t="s">
+      <c r="BJ5" s="53" t="s">
         <v>298</v>
       </c>
-      <c r="BK5" s="52" t="s">
+      <c r="BK5" s="53" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="6" spans="1:63">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="53" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:63">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="53" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:63">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="53" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="9" spans="1:63">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="53" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="10" spans="1:63">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="53" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="11" spans="1:63">
-      <c r="A11" s="52" t="s">
+      <c r="A11" s="53" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="12" spans="1:63">
-      <c r="A12" s="52" t="s">
+      <c r="A12" s="53" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:63">
-      <c r="A13" s="52" t="s">
+      <c r="A13" s="53" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="14" spans="1:63">
-      <c r="A14" s="52" t="s">
+      <c r="A14" s="53" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="15" spans="1:63">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="53" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:63">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="53" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="52" t="s">
+      <c r="A17" s="53" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="52" t="s">
+      <c r="A18" s="53" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="52" t="s">
+      <c r="A19" s="53" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="52" t="s">
+      <c r="A20" s="53" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" s="52" t="s">
+      <c r="A21" s="53" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" s="52" t="s">
+      <c r="A22" s="53" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" s="52" t="s">
+      <c r="A23" s="53" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="52" t="s">
+      <c r="A24" s="53" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="25" spans="1:1">
-      <c r="A25" s="52" t="s">
+      <c r="A25" s="53" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="26" spans="1:1">
-      <c r="A26" s="52" t="s">
+      <c r="A26" s="53" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="27" spans="1:1">
-      <c r="A27" s="52" t="s">
+      <c r="A27" s="53" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="28" spans="1:1">
-      <c r="A28" s="52" t="s">
+      <c r="A28" s="53" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" s="52" t="s">
+      <c r="A29" s="53" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="30" spans="1:1">
-      <c r="A30" s="52" t="s">
+      <c r="A30" s="53" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" s="52" t="s">
+      <c r="A31" s="53" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" s="52" t="s">
+      <c r="A32" s="53" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="53" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="52" t="s">
+      <c r="A34" s="53" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="52" t="s">
+      <c r="A35" s="53" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="52" t="s">
+      <c r="A36" s="53" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="37" spans="1:1">
-      <c r="A37" s="52" t="s">
+      <c r="A37" s="53" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" s="52" t="s">
+      <c r="A38" s="53" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" s="52" t="s">
+      <c r="A39" s="53" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="40" spans="1:1">
-      <c r="A40" s="52" t="s">
+      <c r="A40" s="53" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="41" spans="1:1">
-      <c r="A41" s="52" t="s">
+      <c r="A41" s="53" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="52" t="s">
+      <c r="A42" s="53" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="43" spans="1:1">
-      <c r="A43" s="52" t="s">
+      <c r="A43" s="53" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="44" spans="1:1">
-      <c r="A44" s="52" t="s">
+      <c r="A44" s="53" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="45" spans="1:1">
-      <c r="A45" s="52" t="s">
+      <c r="A45" s="53" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="46" spans="1:1">
-      <c r="A46" s="52" t="s">
+      <c r="A46" s="53" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="47" spans="1:1">
-      <c r="A47" s="52" t="s">
+      <c r="A47" s="53" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="52" t="s">
+      <c r="A48" s="53" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="52" t="s">
+      <c r="A49" s="53" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" s="52" t="s">
+      <c r="A50" s="53" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="52" t="s">
+      <c r="A51" s="53" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="52" spans="1:1">
-      <c r="A52" s="52" t="s">
+      <c r="A52" s="53" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="53" spans="1:1">
-      <c r="A53" s="52" t="s">
+      <c r="A53" s="53" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="54" spans="1:1">
-      <c r="A54" s="52" t="s">
+      <c r="A54" s="53" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" s="52" t="s">
+      <c r="A55" s="53" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="56" spans="1:1">
-      <c r="A56" s="52" t="s">
+      <c r="A56" s="53" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="57" spans="1:1">
-      <c r="A57" s="52" t="s">
+      <c r="A57" s="53" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="58" spans="1:1">
-      <c r="A58" s="52" t="s">
+      <c r="A58" s="53" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="59" spans="1:1">
-      <c r="A59" s="52" t="s">
+      <c r="A59" s="53" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="60" spans="1:1">
-      <c r="A60" s="52" t="s">
+      <c r="A60" s="53" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="61" spans="1:1">
-      <c r="A61" s="52" t="s">
+      <c r="A61" s="53" t="s">
         <v>355</v>
       </c>
     </row>
     <row r="62" spans="1:1">
-      <c r="A62" s="52" t="s">
+      <c r="A62" s="53" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="63" spans="1:1">
-      <c r="A63" s="52" t="s">
+      <c r="A63" s="53" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="64" spans="1:1">
-      <c r="A64" s="52" t="s">
+      <c r="A64" s="53" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="65" spans="1:1">
-      <c r="A65" s="52" t="s">
+      <c r="A65" s="53" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="66" spans="1:1">
-      <c r="A66" s="52" t="s">
+      <c r="A66" s="53" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="67" spans="1:1">
-      <c r="A67" s="52" t="s">
+      <c r="A67" s="53" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="68" spans="1:1">
-      <c r="A68" s="52" t="s">
+      <c r="A68" s="53" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="69" spans="1:1">
-      <c r="A69" s="52" t="s">
+      <c r="A69" s="53" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="70" spans="1:1">
-      <c r="A70" s="52" t="s">
+      <c r="A70" s="53" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="71" spans="1:1">
-      <c r="A71" s="52" t="s">
+      <c r="A71" s="53" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="72" spans="1:1">
-      <c r="A72" s="52" t="s">
+      <c r="A72" s="53" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="73" spans="1:1">
-      <c r="A73" s="52" t="s">
+      <c r="A73" s="53" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="52" t="s">
+      <c r="A74" s="53" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="75" spans="1:1">
-      <c r="A75" s="52" t="s">
+      <c r="A75" s="53" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="76" spans="1:1">
-      <c r="A76" s="52" t="s">
+      <c r="A76" s="53" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="77" spans="1:1">
-      <c r="A77" s="52" t="s">
+      <c r="A77" s="53" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="78" spans="1:1">
-      <c r="A78" s="52" t="s">
+      <c r="A78" s="53" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="79" spans="1:1">
-      <c r="A79" s="52" t="s">
+      <c r="A79" s="53" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="80" spans="1:1">
-      <c r="A80" s="52" t="s">
+      <c r="A80" s="53" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="81" spans="1:1">
-      <c r="A81" s="52" t="s">
+      <c r="A81" s="53" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="82" spans="1:1">
-      <c r="A82" s="52" t="s">
+      <c r="A82" s="53" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="83" spans="1:1">
-      <c r="A83" s="52" t="s">
+      <c r="A83" s="53" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="84" spans="1:1">
-      <c r="A84" s="52" t="s">
+      <c r="A84" s="53" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="85" spans="1:1">
-      <c r="A85" s="52" t="s">
+      <c r="A85" s="53" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="86" spans="1:1">
-      <c r="A86" s="52" t="s">
+      <c r="A86" s="53" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="87" spans="1:1">
-      <c r="A87" s="52" t="s">
+      <c r="A87" s="53" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="88" spans="1:1">
-      <c r="A88" s="52" t="s">
+      <c r="A88" s="53" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="89" spans="1:1">
-      <c r="A89" s="52" t="s">
+      <c r="A89" s="53" t="s">
         <v>383</v>
       </c>
     </row>
     <row r="90" spans="1:1">
-      <c r="A90" s="52" t="s">
+      <c r="A90" s="53" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="91" spans="1:1">
-      <c r="A91" s="52" t="s">
+      <c r="A91" s="53" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="92" spans="1:1">
-      <c r="A92" s="52" t="s">
+      <c r="A92" s="53" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="93" spans="1:1">
-      <c r="A93" s="52" t="s">
+      <c r="A93" s="53" t="s">
         <v>387</v>
       </c>
     </row>
     <row r="94" spans="1:1">
-      <c r="A94" s="52" t="s">
+      <c r="A94" s="53" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="95" spans="1:1">
-      <c r="A95" s="52" t="s">
+      <c r="A95" s="53" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="96" spans="1:1">
-      <c r="A96" s="52" t="s">
+      <c r="A96" s="53" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="97" spans="1:1">
-      <c r="A97" s="52" t="s">
+      <c r="A97" s="53" t="s">
         <v>391</v>
       </c>
     </row>
     <row r="98" spans="1:1">
-      <c r="A98" s="52" t="s">
+      <c r="A98" s="53" t="s">
         <v>392</v>
       </c>
     </row>
     <row r="99" spans="1:1">
-      <c r="A99" s="52" t="s">
+      <c r="A99" s="53" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="100" spans="1:1">
-      <c r="A100" s="52" t="s">
+      <c r="A100" s="53" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="101" spans="1:1">
-      <c r="A101" s="52" t="s">
+      <c r="A101" s="53" t="s">
         <v>395</v>
       </c>
     </row>
     <row r="102" spans="1:1">
-      <c r="A102" s="52" t="s">
+      <c r="A102" s="53" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="103" spans="1:1">
-      <c r="A103" s="52" t="s">
+      <c r="A103" s="53" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="104" spans="1:1">
-      <c r="A104" s="52" t="s">
+      <c r="A104" s="53" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="105" spans="1:1">
-      <c r="A105" s="52" t="s">
+      <c r="A105" s="53" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="106" spans="1:1">
-      <c r="A106" s="52" t="s">
+      <c r="A106" s="53" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="107" spans="1:1">
-      <c r="A107" s="52" t="s">
+      <c r="A107" s="53" t="s">
         <v>401</v>
       </c>
     </row>
     <row r="108" spans="1:1">
-      <c r="A108" s="52" t="s">
+      <c r="A108" s="53" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="109" spans="1:1">
-      <c r="A109" s="52" t="s">
+      <c r="A109" s="53" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="110" spans="1:1">
-      <c r="A110" s="52" t="s">
+      <c r="A110" s="53" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="111" spans="1:1">
-      <c r="A111" s="52" t="s">
+      <c r="A111" s="53" t="s">
         <v>405</v>
       </c>
     </row>
     <row r="112" spans="1:1">
-      <c r="A112" s="52" t="s">
+      <c r="A112" s="53" t="s">
         <v>406</v>
       </c>
     </row>
     <row r="113" spans="1:1">
-      <c r="A113" s="52" t="s">
+      <c r="A113" s="53" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="114" spans="1:1">
-      <c r="A114" s="52" t="s">
+      <c r="A114" s="53" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="115" spans="1:1">
-      <c r="A115" s="52" t="s">
+      <c r="A115" s="53" t="s">
         <v>409</v>
       </c>
     </row>
     <row r="116" spans="1:1">
-      <c r="A116" s="52" t="s">
+      <c r="A116" s="53" t="s">
         <v>410</v>
       </c>
     </row>
     <row r="117" spans="1:1">
-      <c r="A117" s="52" t="s">
+      <c r="A117" s="53" t="s">
         <v>411</v>
       </c>
     </row>
     <row r="118" spans="1:1">
-      <c r="A118" s="52" t="s">
+      <c r="A118" s="53" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="119" spans="1:1">
-      <c r="A119" s="52" t="s">
+      <c r="A119" s="53" t="s">
         <v>413</v>
       </c>
     </row>
     <row r="120" spans="1:1">
-      <c r="A120" s="52" t="s">
+      <c r="A120" s="53" t="s">
         <v>414</v>
       </c>
     </row>
     <row r="121" spans="1:1">
-      <c r="A121" s="52" t="s">
+      <c r="A121" s="53" t="s">
         <v>415</v>
       </c>
     </row>
     <row r="122" spans="1:1">
-      <c r="A122" s="52" t="s">
+      <c r="A122" s="53" t="s">
         <v>416</v>
       </c>
     </row>
     <row r="123" spans="1:1">
-      <c r="A123" s="52" t="s">
+      <c r="A123" s="53" t="s">
         <v>417</v>
       </c>
     </row>
     <row r="124" spans="1:1">
-      <c r="A124" s="52" t="s">
+      <c r="A124" s="53" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="125" spans="1:1">
-      <c r="A125" s="52" t="s">
+      <c r="A125" s="53" t="s">
         <v>419</v>
       </c>
     </row>
     <row r="126" spans="1:1">
-      <c r="A126" s="52" t="s">
+      <c r="A126" s="53" t="s">
         <v>420</v>
       </c>
     </row>
     <row r="127" spans="1:1">
-      <c r="A127" s="52" t="s">
+      <c r="A127" s="53" t="s">
         <v>421</v>
       </c>
     </row>
     <row r="128" spans="1:1">
-      <c r="A128" s="52" t="s">
+      <c r="A128" s="53" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="129" spans="1:1">
-      <c r="A129" s="52" t="s">
+      <c r="A129" s="53" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="130" spans="1:1">
-      <c r="A130" s="52" t="s">
+      <c r="A130" s="53" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="131" spans="1:1">
-      <c r="A131" s="52" t="s">
+      <c r="A131" s="53" t="s">
         <v>425</v>
       </c>
     </row>
     <row r="132" spans="1:1">
-      <c r="A132" s="52" t="s">
+      <c r="A132" s="53" t="s">
         <v>426</v>
       </c>
     </row>
     <row r="133" spans="1:1">
-      <c r="A133" s="52" t="s">
+      <c r="A133" s="53" t="s">
         <v>427</v>
       </c>
     </row>
     <row r="134" spans="1:1">
-      <c r="A134" s="52" t="s">
+      <c r="A134" s="53" t="s">
         <v>428</v>
       </c>
     </row>
     <row r="135" spans="1:1">
-      <c r="A135" s="52" t="s">
+      <c r="A135" s="53" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="136" spans="1:1">
-      <c r="A136" s="52" t="s">
+      <c r="A136" s="53" t="s">
         <v>430</v>
       </c>
     </row>
     <row r="137" spans="1:1">
-      <c r="A137" s="52" t="s">
+      <c r="A137" s="53" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="138" spans="1:1">
-      <c r="A138" s="52" t="s">
+      <c r="A138" s="53" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="139" spans="1:1">
-      <c r="A139" s="52" t="s">
+      <c r="A139" s="53" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="140" spans="1:1">
-      <c r="A140" s="52" t="s">
+      <c r="A140" s="53" t="s">
         <v>434</v>
       </c>
     </row>
     <row r="141" spans="1:1">
-      <c r="A141" s="52" t="s">
+      <c r="A141" s="53" t="s">
         <v>435</v>
       </c>
     </row>
     <row r="142" spans="1:1">
-      <c r="A142" s="52" t="s">
+      <c r="A142" s="53" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="143" spans="1:1">
-      <c r="A143" s="52" t="s">
+      <c r="A143" s="53" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="144" spans="1:1">
-      <c r="A144" s="52" t="s">
+      <c r="A144" s="53" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="145" spans="1:1">
-      <c r="A145" s="52" t="s">
+      <c r="A145" s="53" t="s">
         <v>439</v>
       </c>
     </row>
     <row r="146" spans="1:1">
-      <c r="A146" s="52" t="s">
+      <c r="A146" s="53" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="147" spans="1:1">
-      <c r="A147" s="52" t="s">
+      <c r="A147" s="53" t="s">
         <v>441</v>
       </c>
     </row>
     <row r="148" spans="1:1">
-      <c r="A148" s="52" t="s">
+      <c r="A148" s="53" t="s">
         <v>442</v>
       </c>
     </row>
     <row r="149" spans="1:1">
-      <c r="A149" s="52" t="s">
+      <c r="A149" s="53" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="150" spans="1:1">
-      <c r="A150" s="52" t="s">
+      <c r="A150" s="53" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="151" spans="1:1">
-      <c r="A151" s="52" t="s">
+      <c r="A151" s="53" t="s">
         <v>445</v>
       </c>
     </row>
     <row r="152" spans="1:1">
-      <c r="A152" s="52" t="s">
+      <c r="A152" s="53" t="s">
         <v>446</v>
       </c>
     </row>
     <row r="153" spans="1:1">
-      <c r="A153" s="52" t="s">
+      <c r="A153" s="53" t="s">
         <v>447</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improving Disbursements 3: Now Finally perfect
</commit_message>
<xml_diff>
--- a/src/v2/tests/header_test.xlsx
+++ b/src/v2/tests/header_test.xlsx
@@ -1680,6 +1680,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="dotted">
         <color auto="1"/>
       </left>
@@ -1779,15 +1788,6 @@
         <color auto="1"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="dashed">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -1948,20 +1948,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1969,35 +1969,35 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2036,7 +2036,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2076,18 +2076,18 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -2434,7 +2434,7 @@
         <f>IF($E$2="","Chose your language",VLOOKUP($E$2,Sprachversionen!$B:$BN,27,FALSE))</f>
         <v>0</v>
       </c>
-      <c r="E2" s="32" t="s">
+      <c r="E2" s="20" t="s">
         <v>1</v>
       </c>
       <c r="J2" s="37">
@@ -2457,6 +2457,7 @@
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE))</f>
         <v>0</v>
       </c>
+      <c r="E3" s="20"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
@@ -2481,7 +2482,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="6"/>
-      <c r="D5" s="20"/>
+      <c r="D5" s="21"/>
     </row>
     <row r="6" spans="2:22">
       <c r="B6" s="36">
@@ -2503,7 +2504,7 @@
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
-      <c r="J7" s="21"/>
+      <c r="J7" s="22"/>
     </row>
     <row r="8" spans="2:22">
       <c r="B8" s="36">
@@ -2522,7 +2523,7 @@
       </c>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
-      <c r="J8" s="22"/>
+      <c r="J8" s="23"/>
       <c r="K8" s="1">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,59,FALSE))</f>
         <v>0</v>
@@ -2545,12 +2546,12 @@
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
-      <c r="J9" s="23"/>
+      <c r="J9" s="24"/>
     </row>
     <row r="10" spans="2:22" ht="13.5" customHeight="1"/>
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
-      <c r="B11" s="24"/>
-      <c r="C11" s="25"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="26"/>
       <c r="D11" s="41">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>0</v>
@@ -2639,8 +2640,8 @@
       <c r="V13" s="57"/>
     </row>
     <row r="14" spans="2:22">
-      <c r="B14" s="26"/>
-      <c r="C14" s="27"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="28"/>
       <c r="D14" s="10"/>
       <c r="E14" s="11"/>
       <c r="F14" s="10"/>
@@ -2684,10 +2685,10 @@
       <c r="D15" s="33">
         <v>0</v>
       </c>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="29"/>
-      <c r="H15" s="30"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="31"/>
       <c r="J15" s="58" t="s">
         <v>4</v>
       </c>
@@ -2726,13 +2727,13 @@
       <c r="D16" s="33">
         <v>0</v>
       </c>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
       <c r="G16" s="50">
         <f>IFERROR(F16/D16,0)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="30"/>
+      <c r="H16" s="31"/>
       <c r="J16" s="58" t="s">
         <v>6</v>
       </c>
@@ -2771,13 +2772,13 @@
       <c r="D17" s="33">
         <v>0</v>
       </c>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
       <c r="G17" s="50">
         <f>IFERROR(F17/D17,0)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="30"/>
+      <c r="H17" s="31"/>
       <c r="J17" s="58" t="s">
         <v>8</v>
       </c>
@@ -2816,13 +2817,13 @@
       <c r="D18" s="33">
         <v>0</v>
       </c>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
       <c r="G18" s="50">
         <f>IFERROR(F18/D18,0)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="30"/>
+      <c r="H18" s="31"/>
       <c r="J18" s="58" t="s">
         <v>10</v>
       </c>
@@ -2861,13 +2862,13 @@
       <c r="D19" s="33">
         <v>0</v>
       </c>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
       <c r="G19" s="50">
         <f>IFERROR(F19/D19,0)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="30"/>
+      <c r="H19" s="31"/>
       <c r="J19" s="58" t="s">
         <v>12</v>
       </c>
@@ -2919,7 +2920,7 @@
         <f>IFERROR(INDEX($F$1:$F$1001,ROW())/INDEX($D$1:$D$1001,ROW()),0)</f>
         <v>0</v>
       </c>
-      <c r="H20" s="31"/>
+      <c r="H20" s="32"/>
       <c r="J20" s="58" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Improvements Right Panel Addings some functions
</commit_message>
<xml_diff>
--- a/src/v2/tests/header_test.xlsx
+++ b/src/v2/tests/header_test.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="484">
   <si>
     <t>_de</t>
   </si>
@@ -315,6 +315,9 @@
   </si>
   <si>
     <t>https://www.kindermissionswerk.org/fuer-partner/service</t>
+  </si>
+  <si>
+    <t>Euro</t>
   </si>
   <si>
     <t>AFN</t>
@@ -1793,6 +1796,50 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color auto="1"/>
@@ -1811,50 +1858,6 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1873,7 +1876,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -1991,6 +1994,10 @@
     <xf numFmtId="165" fontId="1" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="165" fontId="1" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -2028,8 +2035,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2040,8 +2048,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -2051,14 +2062,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2090,6 +2098,7 @@
     <xf numFmtId="167" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2410,12 +2419,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22">
-      <c r="B1" s="34" t="str">
+      <c r="B1" s="35" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,2,FALSE))</f>
         <v>F I N A N Z B E R I C H T</v>
       </c>
       <c r="C1" s="2"/>
-      <c r="J1" s="35" t="str">
+      <c r="J1" s="36" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,60,FALSE))</f>
         <v>Tipp:</v>
       </c>
@@ -2430,14 +2439,14 @@
         <v>0</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="36" t="str">
+      <c r="D2" s="37" t="str">
         <f>IF($E$2="","Chose your language",VLOOKUP($E$2,Sprachversionen!$B:$BN,27,FALSE))</f>
         <v>Sprache</v>
       </c>
       <c r="E2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="37" t="str">
+      <c r="J2" s="38" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,61,FALSE))</f>
         <v>Bitte nutzen Sie zum ausfüllen des Finanzberichts unsere Ausfüllhilfe auf unserer Webseite:</v>
       </c>
@@ -2448,12 +2457,12 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="2:22">
-      <c r="B3" s="34" t="str">
+      <c r="B3" s="35" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,3,FALSE))</f>
         <v>ÜBERSICHT ÜBER EINNAHMEN UND AUSGABEN</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="36" t="str">
+      <c r="D3" s="37" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE))</f>
         <v>Lokalwährung</v>
       </c>
@@ -2466,7 +2475,7 @@
       <c r="O3" s="4"/>
     </row>
     <row r="4" spans="2:22" ht="12" customHeight="1">
-      <c r="J4" s="38" t="str">
+      <c r="J4" s="39" t="str">
         <f>HYPERLINK(VLOOKUP($E$2,Sprachversionen!$B:$BN,62,FALSE))</f>
         <v>https://www.kindermissionswerk.org/fuer-partner/service</v>
       </c>
@@ -2477,7 +2486,7 @@
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="2:22">
-      <c r="B5" s="36" t="str">
+      <c r="B5" s="37" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,4,FALSE))</f>
         <v>Projektnummer</v>
       </c>
@@ -2485,7 +2494,7 @@
       <c r="D5" s="21"/>
     </row>
     <row r="6" spans="2:22">
-      <c r="B6" s="36" t="str">
+      <c r="B6" s="37" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,26,FALSE))</f>
         <v>Projekttitel</v>
       </c>
@@ -2507,17 +2516,17 @@
       <c r="J7" s="22"/>
     </row>
     <row r="8" spans="2:22">
-      <c r="B8" s="36" t="str">
+      <c r="B8" s="37" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,5,FALSE))</f>
         <v>Projektlaufzeit</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="39" t="str">
+      <c r="D8" s="40" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E8" s="8"/>
-      <c r="F8" s="39" t="str">
+      <c r="F8" s="40" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2530,17 +2539,17 @@
       </c>
     </row>
     <row r="9" spans="2:22">
-      <c r="B9" s="36" t="str">
+      <c r="B9" s="37" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,6,FALSE))</f>
         <v>Aktueller Berichtszeitraum</v>
       </c>
       <c r="C9" s="6"/>
-      <c r="D9" s="39" t="str">
+      <c r="D9" s="40" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,7,FALSE))</f>
         <v>von (TT MM JJJJ):</v>
       </c>
       <c r="E9" s="8"/>
-      <c r="F9" s="39" t="str">
+      <c r="F9" s="40" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,8,FALSE))</f>
         <v>bis (TT MM JJJJ):</v>
       </c>
@@ -2552,27 +2561,27 @@
     <row r="11" spans="2:22" ht="12.75" customHeight="1">
       <c r="B11" s="25"/>
       <c r="C11" s="26"/>
-      <c r="D11" s="41" t="str">
+      <c r="D11" s="42" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,11,FALSE))</f>
         <v>Bewilligtes Budget</v>
       </c>
-      <c r="E11" s="42" t="str">
+      <c r="E11" s="43" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,12,FALSE))</f>
         <v>Einnahmen im Berichtszeitraum</v>
       </c>
-      <c r="F11" s="41" t="str">
+      <c r="F11" s="42" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,13,FALSE))</f>
         <v>Einnahmen der gesamten Projektlaufzeit</v>
       </c>
-      <c r="G11" s="41" t="str">
+      <c r="G11" s="42" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,14,FALSE))</f>
         <v>% erhaltene Einnahmen</v>
       </c>
-      <c r="H11" s="43" t="str">
+      <c r="H11" s="44" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,15,FALSE))</f>
         <v>Begründung der Budgetüber- oder unterschreitung</v>
       </c>
-      <c r="J11" s="40" t="str">
+      <c r="J11" s="41" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2581,7 +2590,7 @@
       <c r="M11" s="54"/>
       <c r="N11" s="54"/>
       <c r="O11" s="55"/>
-      <c r="Q11" s="40" t="str">
+      <c r="Q11" s="41" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,19,FALSE))</f>
         <v>KMW Mittel*</v>
       </c>
@@ -2592,7 +2601,7 @@
       <c r="V11" s="55"/>
     </row>
     <row r="12" spans="2:22">
-      <c r="B12" s="44" t="str">
+      <c r="B12" s="45" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,9,FALSE))</f>
         <v>EINNAHMEN</v>
       </c>
@@ -2616,7 +2625,7 @@
       <c r="V12" s="57"/>
     </row>
     <row r="13" spans="2:22">
-      <c r="B13" s="45" t="str">
+      <c r="B13" s="46" t="str">
         <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,10,FALSE))</f>
         <v>(in lokaler Währung)</v>
       </c>
@@ -2628,16 +2637,40 @@
       <c r="H13" s="12"/>
       <c r="J13" s="56"/>
       <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="57"/>
+      <c r="L13" s="47" t="str">
+        <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
+        <v>Datum</v>
+      </c>
+      <c r="M13" s="47" t="str">
+        <f>VLOOKUP($E$2,Sprachversionen!$B:$BN,63,FALSE)</f>
+        <v>Euro</v>
+      </c>
+      <c r="N13" s="47" t="str">
+        <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
+        <v>Lokalwährung</v>
+      </c>
+      <c r="O13" s="47" t="str">
+        <f>VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE)</f>
+        <v>WK</v>
+      </c>
       <c r="Q13" s="56"/>
       <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="1"/>
-      <c r="U13" s="1"/>
-      <c r="V13" s="57"/>
+      <c r="S13" s="47" t="str">
+        <f>IF($E$2="","",VLOOKUP($E$2,Sprachversionen!$B:$BN,22,FALSE))</f>
+        <v>Datum</v>
+      </c>
+      <c r="T13" s="47" t="str">
+        <f>VLOOKUP($E$2,Sprachversionen!$B:$BN,63,FALSE)</f>
+        <v>Euro</v>
+      </c>
+      <c r="U13" s="47" t="str">
+        <f>IF(E3="",VLOOKUP($E$2,Sprachversionen!$B:$BN,28,FALSE),E3)</f>
+        <v>Lokalwährung</v>
+      </c>
+      <c r="V13" s="47" t="str">
+        <f>VLOOKUP($E$2,Sprachversionen!$B:$BN,58,FALSE)</f>
+        <v>WK</v>
+      </c>
     </row>
     <row r="14" spans="2:22">
       <c r="B14" s="27"/>
@@ -2682,7 +2715,7 @@
         <v>Saldovortrag (aus vorherigem Berichtszeitraum)</v>
       </c>
       <c r="C15" s="15"/>
-      <c r="D15" s="33">
+      <c r="D15" s="34">
         <v>0</v>
       </c>
       <c r="E15" s="29"/>
@@ -2724,7 +2757,7 @@
         <v>Lokale Eigenleistung</v>
       </c>
       <c r="C16" s="16"/>
-      <c r="D16" s="33">
+      <c r="D16" s="34">
         <v>0</v>
       </c>
       <c r="E16" s="29"/>
@@ -2769,7 +2802,7 @@
         <v>Beiträge von dritter Seite</v>
       </c>
       <c r="C17" s="16"/>
-      <c r="D17" s="33">
+      <c r="D17" s="34">
         <v>0</v>
       </c>
       <c r="E17" s="29"/>
@@ -2814,7 +2847,7 @@
         <v>KMW Mittel*</v>
       </c>
       <c r="C18" s="16"/>
-      <c r="D18" s="33">
+      <c r="D18" s="34">
         <v>0</v>
       </c>
       <c r="E18" s="29"/>
@@ -2859,7 +2892,7 @@
         <v>Zinserträge</v>
       </c>
       <c r="C19" s="16"/>
-      <c r="D19" s="33">
+      <c r="D19" s="34">
         <v>0</v>
       </c>
       <c r="E19" s="29"/>
@@ -3325,1702 +3358,1717 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BK153"/>
+  <dimension ref="A1:BL153"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:63">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:64">
+      <c r="A1" s="68" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="68" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="46" t="s">
+      <c r="E1" s="68" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="46" t="s">
+      <c r="F1" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="46" t="s">
+      <c r="G1" s="68" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="46" t="s">
+      <c r="H1" s="68" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="46" t="s">
+      <c r="I1" s="68" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="46" t="s">
+      <c r="J1" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="46" t="s">
+      <c r="L1" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="46" t="s">
+      <c r="M1" s="68" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="46" t="s">
+      <c r="N1" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="O1" s="46" t="s">
+      <c r="O1" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="46" t="s">
+      <c r="P1" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="46" t="s">
+      <c r="Q1" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="R1" s="46" t="s">
+      <c r="R1" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="S1" s="46" t="s">
+      <c r="S1" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="T1" s="46" t="s">
+      <c r="T1" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="U1" s="46" t="s">
+      <c r="U1" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="V1" s="46" t="s">
+      <c r="V1" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="W1" s="46" t="s">
+      <c r="W1" s="68" t="s">
         <v>59</v>
       </c>
-      <c r="X1" s="46" t="s">
+      <c r="X1" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="Y1" s="46" t="s">
+      <c r="Y1" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="Z1" s="46" t="s">
+      <c r="Z1" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="AA1" s="46" t="s">
+      <c r="AA1" s="68" t="s">
         <v>63</v>
       </c>
-      <c r="AB1" s="46" t="s">
+      <c r="AB1" s="68" t="s">
         <v>64</v>
       </c>
-      <c r="AC1" s="46" t="s">
+      <c r="AC1" s="68" t="s">
         <v>65</v>
       </c>
-      <c r="AD1" s="46" t="s">
+      <c r="AD1" s="68" t="s">
         <v>66</v>
       </c>
-      <c r="AE1" s="46" t="s">
+      <c r="AE1" s="68" t="s">
         <v>67</v>
       </c>
-      <c r="AF1" s="46" t="s">
+      <c r="AF1" s="68" t="s">
         <v>68</v>
       </c>
-      <c r="AG1" s="46" t="s">
+      <c r="AG1" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="AH1" s="46" t="s">
+      <c r="AH1" s="68" t="s">
         <v>70</v>
       </c>
-      <c r="AI1" s="46" t="s">
+      <c r="AI1" s="68" t="s">
         <v>71</v>
       </c>
-      <c r="AJ1" s="46" t="s">
+      <c r="AJ1" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="AK1" s="46" t="s">
+      <c r="AK1" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="AL1" s="46" t="s">
+      <c r="AL1" s="68" t="s">
         <v>74</v>
       </c>
-      <c r="AM1" s="46" t="s">
+      <c r="AM1" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="AN1" s="46" t="s">
+      <c r="AN1" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="AO1" s="46" t="s">
+      <c r="AO1" s="68" t="s">
         <v>77</v>
       </c>
-      <c r="AP1" s="46" t="s">
+      <c r="AP1" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="AQ1" s="46" t="s">
+      <c r="AQ1" s="68" t="s">
         <v>79</v>
       </c>
-      <c r="AR1" s="46" t="s">
+      <c r="AR1" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="AS1" s="46" t="s">
+      <c r="AS1" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="AT1" s="46" t="s">
+      <c r="AT1" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="AU1" s="46" t="s">
+      <c r="AU1" s="68" t="s">
         <v>83</v>
       </c>
-      <c r="AV1" s="46" t="s">
+      <c r="AV1" s="68" t="s">
         <v>84</v>
       </c>
-      <c r="AW1" s="46" t="s">
+      <c r="AW1" s="68" t="s">
         <v>85</v>
       </c>
-      <c r="AX1" s="46" t="s">
+      <c r="AX1" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="AY1" s="46" t="s">
+      <c r="AY1" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="AZ1" s="46" t="s">
+      <c r="AZ1" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="BA1" s="46" t="s">
+      <c r="BA1" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="BB1" s="46" t="s">
+      <c r="BB1" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="BC1" s="46" t="s">
+      <c r="BC1" s="68" t="s">
         <v>91</v>
       </c>
-      <c r="BD1" s="46" t="s">
+      <c r="BD1" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="BE1" s="46" t="s">
+      <c r="BE1" s="68" t="s">
         <v>93</v>
       </c>
-      <c r="BF1" s="46" t="s">
+      <c r="BF1" s="68" t="s">
         <v>94</v>
       </c>
-      <c r="BG1" s="46" t="s">
+      <c r="BG1" s="68" t="s">
         <v>95</v>
       </c>
-      <c r="BH1" s="46" t="s">
+      <c r="BH1" s="68" t="s">
         <v>96</v>
       </c>
-      <c r="BI1" s="46" t="s">
+      <c r="BI1" s="68" t="s">
         <v>97</v>
       </c>
-      <c r="BJ1" s="46" t="s">
+      <c r="BJ1" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="BK1" s="46" t="s">
+      <c r="BK1" s="68" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="2" spans="1:63">
-      <c r="A2" s="46" t="s">
+      <c r="BL1" s="68" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="46" t="s">
+    </row>
+    <row r="2" spans="1:64">
+      <c r="A2" s="68" t="s">
         <v>101</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="B2" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="C2" s="68" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="D2" s="68" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="46" t="s">
+      <c r="E2" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="G2" s="46" t="s">
+      <c r="F2" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="46" t="s">
+      <c r="G2" s="68" t="s">
         <v>107</v>
       </c>
-      <c r="I2" s="46" t="s">
+      <c r="H2" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="46" t="s">
+      <c r="I2" s="68" t="s">
         <v>109</v>
       </c>
-      <c r="K2" s="46" t="s">
+      <c r="J2" s="68" t="s">
         <v>110</v>
       </c>
-      <c r="L2" s="46" t="s">
+      <c r="K2" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="M2" s="46" t="s">
+      <c r="L2" s="68" t="s">
         <v>112</v>
       </c>
-      <c r="N2" s="46" t="s">
+      <c r="M2" s="68" t="s">
         <v>113</v>
       </c>
-      <c r="O2" s="46" t="s">
+      <c r="N2" s="68" t="s">
         <v>114</v>
       </c>
-      <c r="P2" s="46" t="s">
+      <c r="O2" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="Q2" s="46" t="s">
+      <c r="P2" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="R2" s="46" t="s">
+      <c r="Q2" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="S2" s="46" t="s">
+      <c r="R2" s="68" t="s">
         <v>118</v>
       </c>
-      <c r="T2" s="46" t="s">
+      <c r="S2" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="U2" s="46" t="s">
+      <c r="T2" s="68" t="s">
         <v>120</v>
       </c>
-      <c r="V2" s="46" t="s">
+      <c r="U2" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="W2" s="46" t="s">
+      <c r="V2" s="68" t="s">
         <v>122</v>
       </c>
-      <c r="X2" s="46" t="s">
+      <c r="W2" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="Y2" s="46" t="s">
+      <c r="X2" s="68" t="s">
         <v>124</v>
       </c>
-      <c r="Z2" s="46" t="s">
+      <c r="Y2" s="68" t="s">
         <v>125</v>
       </c>
-      <c r="AA2" s="46" t="s">
+      <c r="Z2" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="AB2" s="46" t="s">
+      <c r="AA2" s="68" t="s">
         <v>127</v>
       </c>
-      <c r="AC2" s="46" t="s">
+      <c r="AB2" s="68" t="s">
         <v>128</v>
       </c>
-      <c r="AD2" s="46" t="s">
+      <c r="AC2" s="68" t="s">
         <v>129</v>
       </c>
-      <c r="AE2" s="46" t="s">
+      <c r="AD2" s="68" t="s">
         <v>130</v>
       </c>
-      <c r="AF2" s="46" t="s">
+      <c r="AE2" s="68" t="s">
         <v>131</v>
       </c>
-      <c r="AG2" s="46" t="s">
+      <c r="AF2" s="68" t="s">
         <v>132</v>
       </c>
-      <c r="AH2" s="46" t="s">
+      <c r="AG2" s="68" t="s">
         <v>133</v>
       </c>
-      <c r="AI2" s="46" t="s">
+      <c r="AH2" s="68" t="s">
         <v>134</v>
       </c>
-      <c r="AJ2" s="46" t="s">
+      <c r="AI2" s="68" t="s">
         <v>135</v>
       </c>
-      <c r="AK2" s="46" t="s">
+      <c r="AJ2" s="68" t="s">
         <v>136</v>
       </c>
-      <c r="AL2" s="46" t="s">
+      <c r="AK2" s="68" t="s">
         <v>137</v>
       </c>
-      <c r="AM2" s="46" t="s">
+      <c r="AL2" s="68" t="s">
         <v>138</v>
       </c>
-      <c r="AN2" s="46" t="s">
+      <c r="AM2" s="68" t="s">
         <v>139</v>
       </c>
-      <c r="AO2" s="46" t="s">
+      <c r="AN2" s="68" t="s">
+        <v>140</v>
+      </c>
+      <c r="AO2" s="68" t="s">
         <v>77</v>
       </c>
-      <c r="AP2" s="46" t="s">
+      <c r="AP2" s="68" t="s">
+        <v>141</v>
+      </c>
+      <c r="AQ2" s="68" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR2" s="68" t="s">
+        <v>142</v>
+      </c>
+      <c r="AS2" s="68" t="s">
+        <v>143</v>
+      </c>
+      <c r="AT2" s="68" t="s">
+        <v>144</v>
+      </c>
+      <c r="AU2" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="AV2" s="68" t="s">
+        <v>84</v>
+      </c>
+      <c r="AW2" s="68" t="s">
+        <v>146</v>
+      </c>
+      <c r="AX2" s="68" t="s">
+        <v>147</v>
+      </c>
+      <c r="AY2" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="AZ2" s="68" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA2" s="68" t="s">
+        <v>150</v>
+      </c>
+      <c r="BB2" s="68" t="s">
+        <v>151</v>
+      </c>
+      <c r="BC2" s="68" t="s">
+        <v>152</v>
+      </c>
+      <c r="BD2" s="68" t="s">
+        <v>153</v>
+      </c>
+      <c r="BE2" s="68" t="s">
+        <v>154</v>
+      </c>
+      <c r="BF2" s="68" t="s">
+        <v>155</v>
+      </c>
+      <c r="BG2" s="68" t="s">
+        <v>156</v>
+      </c>
+      <c r="BH2" s="68" t="s">
+        <v>157</v>
+      </c>
+      <c r="BI2" s="68" t="s">
+        <v>158</v>
+      </c>
+      <c r="BJ2" s="68" t="s">
+        <v>159</v>
+      </c>
+      <c r="BK2" s="68" t="s">
+        <v>160</v>
+      </c>
+      <c r="BL2" s="68" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:64">
+      <c r="A3" s="68" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="68" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" s="68" t="s">
+        <v>164</v>
+      </c>
+      <c r="E3" s="68" t="s">
+        <v>165</v>
+      </c>
+      <c r="F3" s="68" t="s">
+        <v>166</v>
+      </c>
+      <c r="G3" s="68" t="s">
+        <v>167</v>
+      </c>
+      <c r="H3" s="68" t="s">
+        <v>168</v>
+      </c>
+      <c r="I3" s="68" t="s">
+        <v>168</v>
+      </c>
+      <c r="J3" s="68" t="s">
+        <v>169</v>
+      </c>
+      <c r="K3" s="68" t="s">
+        <v>170</v>
+      </c>
+      <c r="L3" s="68" t="s">
+        <v>171</v>
+      </c>
+      <c r="M3" s="68" t="s">
+        <v>172</v>
+      </c>
+      <c r="N3" s="68" t="s">
+        <v>173</v>
+      </c>
+      <c r="O3" s="68" t="s">
+        <v>174</v>
+      </c>
+      <c r="P3" s="68" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q3" s="68" t="s">
+        <v>176</v>
+      </c>
+      <c r="R3" s="68" t="s">
+        <v>177</v>
+      </c>
+      <c r="S3" s="68" t="s">
+        <v>178</v>
+      </c>
+      <c r="T3" s="68" t="s">
+        <v>179</v>
+      </c>
+      <c r="U3" s="68" t="s">
+        <v>180</v>
+      </c>
+      <c r="V3" s="68" t="s">
+        <v>181</v>
+      </c>
+      <c r="W3" s="68" t="s">
+        <v>123</v>
+      </c>
+      <c r="X3" s="68" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y3" s="68" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z3" s="68" t="s">
+        <v>184</v>
+      </c>
+      <c r="AA3" s="68" t="s">
+        <v>185</v>
+      </c>
+      <c r="AB3" s="68" t="s">
+        <v>186</v>
+      </c>
+      <c r="AC3" s="68" t="s">
+        <v>187</v>
+      </c>
+      <c r="AD3" s="68" t="s">
+        <v>188</v>
+      </c>
+      <c r="AE3" s="68" t="s">
+        <v>189</v>
+      </c>
+      <c r="AF3" s="68" t="s">
+        <v>190</v>
+      </c>
+      <c r="AG3" s="68" t="s">
+        <v>191</v>
+      </c>
+      <c r="AH3" s="68" t="s">
+        <v>192</v>
+      </c>
+      <c r="AI3" s="68" t="s">
+        <v>193</v>
+      </c>
+      <c r="AJ3" s="68" t="s">
+        <v>194</v>
+      </c>
+      <c r="AK3" s="68" t="s">
+        <v>195</v>
+      </c>
+      <c r="AL3" s="68" t="s">
+        <v>196</v>
+      </c>
+      <c r="AM3" s="68" t="s">
+        <v>197</v>
+      </c>
+      <c r="AN3" s="68" t="s">
         <v>140</v>
       </c>
-      <c r="AQ2" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="AR2" s="46" t="s">
-        <v>141</v>
-      </c>
-      <c r="AS2" s="46" t="s">
-        <v>142</v>
-      </c>
-      <c r="AT2" s="46" t="s">
-        <v>143</v>
-      </c>
-      <c r="AU2" s="46" t="s">
-        <v>144</v>
-      </c>
-      <c r="AV2" s="46" t="s">
-        <v>84</v>
-      </c>
-      <c r="AW2" s="46" t="s">
-        <v>145</v>
-      </c>
-      <c r="AX2" s="46" t="s">
-        <v>146</v>
-      </c>
-      <c r="AY2" s="46" t="s">
-        <v>147</v>
-      </c>
-      <c r="AZ2" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="BA2" s="46" t="s">
-        <v>149</v>
-      </c>
-      <c r="BB2" s="46" t="s">
-        <v>150</v>
-      </c>
-      <c r="BC2" s="46" t="s">
-        <v>151</v>
-      </c>
-      <c r="BD2" s="46" t="s">
-        <v>152</v>
-      </c>
-      <c r="BE2" s="46" t="s">
-        <v>153</v>
-      </c>
-      <c r="BF2" s="46" t="s">
-        <v>154</v>
-      </c>
-      <c r="BG2" s="46" t="s">
-        <v>155</v>
-      </c>
-      <c r="BH2" s="46" t="s">
-        <v>156</v>
-      </c>
-      <c r="BI2" s="46" t="s">
-        <v>157</v>
-      </c>
-      <c r="BJ2" s="46" t="s">
-        <v>158</v>
-      </c>
-      <c r="BK2" s="46" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="3" spans="1:63">
-      <c r="A3" s="46" t="s">
-        <v>160</v>
-      </c>
-      <c r="B3" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="C3" s="46" t="s">
-        <v>162</v>
-      </c>
-      <c r="D3" s="46" t="s">
-        <v>163</v>
-      </c>
-      <c r="E3" s="46" t="s">
-        <v>164</v>
-      </c>
-      <c r="F3" s="46" t="s">
-        <v>165</v>
-      </c>
-      <c r="G3" s="46" t="s">
-        <v>166</v>
-      </c>
-      <c r="H3" s="46" t="s">
-        <v>167</v>
-      </c>
-      <c r="I3" s="46" t="s">
-        <v>167</v>
-      </c>
-      <c r="J3" s="46" t="s">
-        <v>168</v>
-      </c>
-      <c r="K3" s="46" t="s">
-        <v>169</v>
-      </c>
-      <c r="L3" s="46" t="s">
-        <v>170</v>
-      </c>
-      <c r="M3" s="46" t="s">
-        <v>171</v>
-      </c>
-      <c r="N3" s="46" t="s">
-        <v>172</v>
-      </c>
-      <c r="O3" s="46" t="s">
-        <v>173</v>
-      </c>
-      <c r="P3" s="46" t="s">
-        <v>174</v>
-      </c>
-      <c r="Q3" s="46" t="s">
-        <v>175</v>
-      </c>
-      <c r="R3" s="46" t="s">
-        <v>176</v>
-      </c>
-      <c r="S3" s="46" t="s">
-        <v>177</v>
-      </c>
-      <c r="T3" s="46" t="s">
-        <v>178</v>
-      </c>
-      <c r="U3" s="46" t="s">
-        <v>179</v>
-      </c>
-      <c r="V3" s="46" t="s">
-        <v>180</v>
-      </c>
-      <c r="W3" s="46" t="s">
+      <c r="AO3" s="68" t="s">
+        <v>77</v>
+      </c>
+      <c r="AP3" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="AQ3" s="68" t="s">
+        <v>181</v>
+      </c>
+      <c r="AR3" s="68" t="s">
+        <v>199</v>
+      </c>
+      <c r="AS3" s="68" t="s">
+        <v>200</v>
+      </c>
+      <c r="AT3" s="68" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU3" s="68" t="s">
+        <v>202</v>
+      </c>
+      <c r="AV3" s="68" t="s">
+        <v>203</v>
+      </c>
+      <c r="AW3" s="68" t="s">
+        <v>204</v>
+      </c>
+      <c r="AX3" s="68" t="s">
+        <v>205</v>
+      </c>
+      <c r="AY3" s="68" t="s">
+        <v>206</v>
+      </c>
+      <c r="AZ3" s="68" t="s">
+        <v>207</v>
+      </c>
+      <c r="BA3" s="68" t="s">
+        <v>208</v>
+      </c>
+      <c r="BB3" s="68" t="s">
+        <v>209</v>
+      </c>
+      <c r="BC3" s="68" t="s">
+        <v>210</v>
+      </c>
+      <c r="BD3" s="68" t="s">
+        <v>211</v>
+      </c>
+      <c r="BE3" s="68" t="s">
+        <v>212</v>
+      </c>
+      <c r="BF3" s="68" t="s">
+        <v>213</v>
+      </c>
+      <c r="BG3" s="68" t="s">
+        <v>214</v>
+      </c>
+      <c r="BH3" s="68" t="s">
+        <v>215</v>
+      </c>
+      <c r="BI3" s="68" t="s">
+        <v>216</v>
+      </c>
+      <c r="BJ3" s="68" t="s">
+        <v>217</v>
+      </c>
+      <c r="BK3" s="68" t="s">
+        <v>218</v>
+      </c>
+      <c r="BL3" s="68" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:64">
+      <c r="A4" s="68" t="s">
+        <v>219</v>
+      </c>
+      <c r="B4" s="68" t="s">
+        <v>220</v>
+      </c>
+      <c r="C4" s="68" t="s">
+        <v>221</v>
+      </c>
+      <c r="D4" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="E4" s="68" t="s">
+        <v>223</v>
+      </c>
+      <c r="F4" s="68" t="s">
+        <v>224</v>
+      </c>
+      <c r="G4" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="H4" s="68" t="s">
+        <v>226</v>
+      </c>
+      <c r="I4" s="68" t="s">
+        <v>227</v>
+      </c>
+      <c r="J4" s="68" t="s">
+        <v>228</v>
+      </c>
+      <c r="K4" s="68" t="s">
+        <v>229</v>
+      </c>
+      <c r="L4" s="68" t="s">
+        <v>230</v>
+      </c>
+      <c r="M4" s="68" t="s">
+        <v>231</v>
+      </c>
+      <c r="N4" s="68" t="s">
+        <v>232</v>
+      </c>
+      <c r="O4" s="68" t="s">
+        <v>233</v>
+      </c>
+      <c r="P4" s="68" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q4" s="68" t="s">
+        <v>235</v>
+      </c>
+      <c r="R4" s="68" t="s">
+        <v>236</v>
+      </c>
+      <c r="S4" s="68" t="s">
+        <v>237</v>
+      </c>
+      <c r="T4" s="68" t="s">
+        <v>238</v>
+      </c>
+      <c r="U4" s="68" t="s">
+        <v>239</v>
+      </c>
+      <c r="V4" s="68" t="s">
+        <v>181</v>
+      </c>
+      <c r="W4" s="68" t="s">
+        <v>240</v>
+      </c>
+      <c r="X4" s="68" t="s">
+        <v>241</v>
+      </c>
+      <c r="Y4" s="68" t="s">
+        <v>242</v>
+      </c>
+      <c r="Z4" s="68" t="s">
+        <v>243</v>
+      </c>
+      <c r="AA4" s="68" t="s">
+        <v>244</v>
+      </c>
+      <c r="AB4" s="68" t="s">
+        <v>245</v>
+      </c>
+      <c r="AC4" s="68" t="s">
+        <v>246</v>
+      </c>
+      <c r="AD4" s="68" t="s">
+        <v>247</v>
+      </c>
+      <c r="AE4" s="68" t="s">
+        <v>248</v>
+      </c>
+      <c r="AF4" s="68" t="s">
+        <v>249</v>
+      </c>
+      <c r="AG4" s="68" t="s">
+        <v>250</v>
+      </c>
+      <c r="AH4" s="68" t="s">
+        <v>251</v>
+      </c>
+      <c r="AI4" s="68" t="s">
+        <v>252</v>
+      </c>
+      <c r="AJ4" s="68" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK4" s="68" t="s">
+        <v>254</v>
+      </c>
+      <c r="AL4" s="68" t="s">
+        <v>255</v>
+      </c>
+      <c r="AM4" s="68" t="s">
+        <v>256</v>
+      </c>
+      <c r="AN4" s="68" t="s">
+        <v>257</v>
+      </c>
+      <c r="AO4" s="68" t="s">
+        <v>258</v>
+      </c>
+      <c r="AP4" s="68" t="s">
+        <v>259</v>
+      </c>
+      <c r="AQ4" s="68" t="s">
         <v>122</v>
       </c>
-      <c r="X3" s="46" t="s">
+      <c r="AR4" s="68" t="s">
+        <v>260</v>
+      </c>
+      <c r="AS4" s="68" t="s">
+        <v>261</v>
+      </c>
+      <c r="AT4" s="68" t="s">
+        <v>262</v>
+      </c>
+      <c r="AU4" s="68" t="s">
+        <v>263</v>
+      </c>
+      <c r="AV4" s="68" t="s">
+        <v>264</v>
+      </c>
+      <c r="AW4" s="68" t="s">
+        <v>265</v>
+      </c>
+      <c r="AX4" s="68" t="s">
+        <v>266</v>
+      </c>
+      <c r="AY4" s="68" t="s">
+        <v>267</v>
+      </c>
+      <c r="AZ4" s="68" t="s">
+        <v>268</v>
+      </c>
+      <c r="BA4" s="68" t="s">
+        <v>269</v>
+      </c>
+      <c r="BB4" s="68" t="s">
+        <v>270</v>
+      </c>
+      <c r="BC4" s="68" t="s">
+        <v>271</v>
+      </c>
+      <c r="BD4" s="68" t="s">
+        <v>272</v>
+      </c>
+      <c r="BE4" s="68" t="s">
+        <v>273</v>
+      </c>
+      <c r="BF4" s="68" t="s">
+        <v>274</v>
+      </c>
+      <c r="BG4" s="68" t="s">
+        <v>214</v>
+      </c>
+      <c r="BH4" s="68" t="s">
+        <v>275</v>
+      </c>
+      <c r="BI4" s="68" t="s">
+        <v>276</v>
+      </c>
+      <c r="BJ4" s="68" t="s">
+        <v>277</v>
+      </c>
+      <c r="BK4" s="68" t="s">
+        <v>278</v>
+      </c>
+      <c r="BL4" s="68" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:64">
+      <c r="A5" s="68" t="s">
+        <v>279</v>
+      </c>
+      <c r="B5" s="68" t="s">
+        <v>280</v>
+      </c>
+      <c r="C5" s="68" t="s">
+        <v>281</v>
+      </c>
+      <c r="D5" s="68" t="s">
+        <v>282</v>
+      </c>
+      <c r="E5" s="68" t="s">
+        <v>283</v>
+      </c>
+      <c r="F5" s="68" t="s">
+        <v>284</v>
+      </c>
+      <c r="G5" s="68" t="s">
+        <v>285</v>
+      </c>
+      <c r="H5" s="68" t="s">
+        <v>226</v>
+      </c>
+      <c r="I5" s="68" t="s">
+        <v>286</v>
+      </c>
+      <c r="J5" s="68" t="s">
+        <v>287</v>
+      </c>
+      <c r="K5" s="68" t="s">
+        <v>288</v>
+      </c>
+      <c r="L5" s="68" t="s">
+        <v>289</v>
+      </c>
+      <c r="M5" s="68" t="s">
+        <v>290</v>
+      </c>
+      <c r="N5" s="68" t="s">
+        <v>291</v>
+      </c>
+      <c r="O5" s="68" t="s">
+        <v>292</v>
+      </c>
+      <c r="P5" s="68" t="s">
+        <v>293</v>
+      </c>
+      <c r="Q5" s="68" t="s">
+        <v>294</v>
+      </c>
+      <c r="R5" s="68" t="s">
+        <v>295</v>
+      </c>
+      <c r="S5" s="68" t="s">
+        <v>296</v>
+      </c>
+      <c r="T5" s="68" t="s">
+        <v>297</v>
+      </c>
+      <c r="U5" s="68" t="s">
+        <v>298</v>
+      </c>
+      <c r="V5" s="68" t="s">
         <v>181</v>
       </c>
-      <c r="Y3" s="46" t="s">
-        <v>182</v>
-      </c>
-      <c r="Z3" s="46" t="s">
-        <v>183</v>
-      </c>
-      <c r="AA3" s="46" t="s">
-        <v>184</v>
-      </c>
-      <c r="AB3" s="46" t="s">
-        <v>185</v>
-      </c>
-      <c r="AC3" s="46" t="s">
-        <v>186</v>
-      </c>
-      <c r="AD3" s="46" t="s">
-        <v>187</v>
-      </c>
-      <c r="AE3" s="46" t="s">
-        <v>188</v>
-      </c>
-      <c r="AF3" s="46" t="s">
-        <v>189</v>
-      </c>
-      <c r="AG3" s="46" t="s">
-        <v>190</v>
-      </c>
-      <c r="AH3" s="46" t="s">
-        <v>191</v>
-      </c>
-      <c r="AI3" s="46" t="s">
-        <v>192</v>
-      </c>
-      <c r="AJ3" s="46" t="s">
-        <v>193</v>
-      </c>
-      <c r="AK3" s="46" t="s">
-        <v>194</v>
-      </c>
-      <c r="AL3" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="AM3" s="46" t="s">
-        <v>196</v>
-      </c>
-      <c r="AN3" s="46" t="s">
-        <v>139</v>
-      </c>
-      <c r="AO3" s="46" t="s">
-        <v>77</v>
-      </c>
-      <c r="AP3" s="46" t="s">
-        <v>197</v>
-      </c>
-      <c r="AQ3" s="46" t="s">
-        <v>180</v>
-      </c>
-      <c r="AR3" s="46" t="s">
-        <v>198</v>
-      </c>
-      <c r="AS3" s="46" t="s">
-        <v>199</v>
-      </c>
-      <c r="AT3" s="46" t="s">
-        <v>200</v>
-      </c>
-      <c r="AU3" s="46" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV3" s="46" t="s">
-        <v>202</v>
-      </c>
-      <c r="AW3" s="46" t="s">
-        <v>203</v>
-      </c>
-      <c r="AX3" s="46" t="s">
-        <v>204</v>
-      </c>
-      <c r="AY3" s="46" t="s">
-        <v>205</v>
-      </c>
-      <c r="AZ3" s="46" t="s">
-        <v>206</v>
-      </c>
-      <c r="BA3" s="46" t="s">
-        <v>207</v>
-      </c>
-      <c r="BB3" s="46" t="s">
-        <v>208</v>
-      </c>
-      <c r="BC3" s="46" t="s">
-        <v>209</v>
-      </c>
-      <c r="BD3" s="46" t="s">
-        <v>210</v>
-      </c>
-      <c r="BE3" s="46" t="s">
-        <v>211</v>
-      </c>
-      <c r="BF3" s="46" t="s">
-        <v>212</v>
-      </c>
-      <c r="BG3" s="46" t="s">
-        <v>213</v>
-      </c>
-      <c r="BH3" s="46" t="s">
+      <c r="W5" s="68" t="s">
+        <v>299</v>
+      </c>
+      <c r="X5" s="68" t="s">
+        <v>300</v>
+      </c>
+      <c r="Y5" s="68" t="s">
+        <v>301</v>
+      </c>
+      <c r="Z5" s="68" t="s">
+        <v>302</v>
+      </c>
+      <c r="AA5" s="68" t="s">
+        <v>303</v>
+      </c>
+      <c r="AB5" s="68" t="s">
+        <v>245</v>
+      </c>
+      <c r="AC5" s="68" t="s">
+        <v>304</v>
+      </c>
+      <c r="AD5" s="68" t="s">
+        <v>305</v>
+      </c>
+      <c r="AE5" s="68" t="s">
+        <v>306</v>
+      </c>
+      <c r="AF5" s="68" t="s">
+        <v>307</v>
+      </c>
+      <c r="AG5" s="68" t="s">
+        <v>308</v>
+      </c>
+      <c r="AH5" s="68" t="s">
+        <v>309</v>
+      </c>
+      <c r="AI5" s="68" t="s">
+        <v>310</v>
+      </c>
+      <c r="AJ5" s="68" t="s">
+        <v>311</v>
+      </c>
+      <c r="AK5" s="68" t="s">
+        <v>312</v>
+      </c>
+      <c r="AL5" s="68" t="s">
+        <v>313</v>
+      </c>
+      <c r="AM5" s="68" t="s">
+        <v>314</v>
+      </c>
+      <c r="AN5" s="68" t="s">
+        <v>315</v>
+      </c>
+      <c r="AO5" s="68" t="s">
+        <v>316</v>
+      </c>
+      <c r="AP5" s="68" t="s">
+        <v>317</v>
+      </c>
+      <c r="AQ5" s="68" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR5" s="68" t="s">
+        <v>318</v>
+      </c>
+      <c r="AS5" s="68" t="s">
+        <v>319</v>
+      </c>
+      <c r="AT5" s="68" t="s">
+        <v>320</v>
+      </c>
+      <c r="AU5" s="68" t="s">
+        <v>321</v>
+      </c>
+      <c r="AV5" s="68" t="s">
+        <v>264</v>
+      </c>
+      <c r="AW5" s="68" t="s">
+        <v>322</v>
+      </c>
+      <c r="AX5" s="68" t="s">
+        <v>323</v>
+      </c>
+      <c r="AY5" s="68" t="s">
+        <v>324</v>
+      </c>
+      <c r="AZ5" s="68" t="s">
+        <v>325</v>
+      </c>
+      <c r="BA5" s="68" t="s">
+        <v>326</v>
+      </c>
+      <c r="BB5" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="BC5" s="68" t="s">
+        <v>328</v>
+      </c>
+      <c r="BD5" s="68" t="s">
+        <v>329</v>
+      </c>
+      <c r="BE5" s="68" t="s">
+        <v>330</v>
+      </c>
+      <c r="BF5" s="68" t="s">
+        <v>331</v>
+      </c>
+      <c r="BG5" s="68" t="s">
         <v>214</v>
       </c>
-      <c r="BI3" s="46" t="s">
-        <v>215</v>
-      </c>
-      <c r="BJ3" s="46" t="s">
-        <v>216</v>
-      </c>
-      <c r="BK3" s="46" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="4" spans="1:63">
-      <c r="A4" s="46" t="s">
-        <v>218</v>
-      </c>
-      <c r="B4" s="46" t="s">
-        <v>219</v>
-      </c>
-      <c r="C4" s="46" t="s">
-        <v>220</v>
-      </c>
-      <c r="D4" s="46" t="s">
-        <v>221</v>
-      </c>
-      <c r="E4" s="46" t="s">
-        <v>222</v>
-      </c>
-      <c r="F4" s="46" t="s">
-        <v>223</v>
-      </c>
-      <c r="G4" s="46" t="s">
-        <v>224</v>
-      </c>
-      <c r="H4" s="46" t="s">
-        <v>225</v>
-      </c>
-      <c r="I4" s="46" t="s">
-        <v>226</v>
-      </c>
-      <c r="J4" s="46" t="s">
-        <v>227</v>
-      </c>
-      <c r="K4" s="46" t="s">
-        <v>228</v>
-      </c>
-      <c r="L4" s="46" t="s">
-        <v>229</v>
-      </c>
-      <c r="M4" s="46" t="s">
-        <v>230</v>
-      </c>
-      <c r="N4" s="46" t="s">
-        <v>231</v>
-      </c>
-      <c r="O4" s="46" t="s">
-        <v>232</v>
-      </c>
-      <c r="P4" s="46" t="s">
-        <v>233</v>
-      </c>
-      <c r="Q4" s="46" t="s">
-        <v>234</v>
-      </c>
-      <c r="R4" s="46" t="s">
-        <v>235</v>
-      </c>
-      <c r="S4" s="46" t="s">
-        <v>236</v>
-      </c>
-      <c r="T4" s="46" t="s">
-        <v>237</v>
-      </c>
-      <c r="U4" s="46" t="s">
-        <v>238</v>
-      </c>
-      <c r="V4" s="46" t="s">
-        <v>180</v>
-      </c>
-      <c r="W4" s="46" t="s">
-        <v>239</v>
-      </c>
-      <c r="X4" s="46" t="s">
-        <v>240</v>
-      </c>
-      <c r="Y4" s="46" t="s">
-        <v>241</v>
-      </c>
-      <c r="Z4" s="46" t="s">
-        <v>242</v>
-      </c>
-      <c r="AA4" s="46" t="s">
-        <v>243</v>
-      </c>
-      <c r="AB4" s="46" t="s">
-        <v>244</v>
-      </c>
-      <c r="AC4" s="46" t="s">
-        <v>245</v>
-      </c>
-      <c r="AD4" s="46" t="s">
-        <v>246</v>
-      </c>
-      <c r="AE4" s="46" t="s">
-        <v>247</v>
-      </c>
-      <c r="AF4" s="46" t="s">
-        <v>248</v>
-      </c>
-      <c r="AG4" s="46" t="s">
-        <v>249</v>
-      </c>
-      <c r="AH4" s="46" t="s">
-        <v>250</v>
-      </c>
-      <c r="AI4" s="46" t="s">
-        <v>251</v>
-      </c>
-      <c r="AJ4" s="46" t="s">
-        <v>252</v>
-      </c>
-      <c r="AK4" s="46" t="s">
-        <v>253</v>
-      </c>
-      <c r="AL4" s="46" t="s">
-        <v>254</v>
-      </c>
-      <c r="AM4" s="46" t="s">
-        <v>255</v>
-      </c>
-      <c r="AN4" s="46" t="s">
-        <v>256</v>
-      </c>
-      <c r="AO4" s="46" t="s">
-        <v>257</v>
-      </c>
-      <c r="AP4" s="46" t="s">
-        <v>258</v>
-      </c>
-      <c r="AQ4" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="AR4" s="46" t="s">
-        <v>259</v>
-      </c>
-      <c r="AS4" s="46" t="s">
-        <v>260</v>
-      </c>
-      <c r="AT4" s="46" t="s">
-        <v>261</v>
-      </c>
-      <c r="AU4" s="46" t="s">
-        <v>262</v>
-      </c>
-      <c r="AV4" s="46" t="s">
-        <v>263</v>
-      </c>
-      <c r="AW4" s="46" t="s">
-        <v>264</v>
-      </c>
-      <c r="AX4" s="46" t="s">
-        <v>265</v>
-      </c>
-      <c r="AY4" s="46" t="s">
-        <v>266</v>
-      </c>
-      <c r="AZ4" s="46" t="s">
-        <v>267</v>
-      </c>
-      <c r="BA4" s="46" t="s">
-        <v>268</v>
-      </c>
-      <c r="BB4" s="46" t="s">
-        <v>269</v>
-      </c>
-      <c r="BC4" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="BD4" s="46" t="s">
-        <v>271</v>
-      </c>
-      <c r="BE4" s="46" t="s">
-        <v>272</v>
-      </c>
-      <c r="BF4" s="46" t="s">
-        <v>273</v>
-      </c>
-      <c r="BG4" s="46" t="s">
-        <v>213</v>
-      </c>
-      <c r="BH4" s="46" t="s">
-        <v>274</v>
-      </c>
-      <c r="BI4" s="46" t="s">
-        <v>275</v>
-      </c>
-      <c r="BJ4" s="46" t="s">
-        <v>276</v>
-      </c>
-      <c r="BK4" s="46" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="5" spans="1:63">
-      <c r="A5" s="46" t="s">
-        <v>278</v>
-      </c>
-      <c r="B5" s="46" t="s">
-        <v>279</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>280</v>
-      </c>
-      <c r="D5" s="46" t="s">
-        <v>281</v>
-      </c>
-      <c r="E5" s="46" t="s">
-        <v>282</v>
-      </c>
-      <c r="F5" s="46" t="s">
-        <v>283</v>
-      </c>
-      <c r="G5" s="46" t="s">
-        <v>284</v>
-      </c>
-      <c r="H5" s="46" t="s">
-        <v>225</v>
-      </c>
-      <c r="I5" s="46" t="s">
-        <v>285</v>
-      </c>
-      <c r="J5" s="46" t="s">
-        <v>286</v>
-      </c>
-      <c r="K5" s="46" t="s">
-        <v>287</v>
-      </c>
-      <c r="L5" s="46" t="s">
-        <v>288</v>
-      </c>
-      <c r="M5" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="N5" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="O5" s="46" t="s">
-        <v>291</v>
-      </c>
-      <c r="P5" s="46" t="s">
-        <v>292</v>
-      </c>
-      <c r="Q5" s="46" t="s">
-        <v>293</v>
-      </c>
-      <c r="R5" s="46" t="s">
-        <v>294</v>
-      </c>
-      <c r="S5" s="46" t="s">
-        <v>295</v>
-      </c>
-      <c r="T5" s="46" t="s">
-        <v>296</v>
-      </c>
-      <c r="U5" s="46" t="s">
-        <v>297</v>
-      </c>
-      <c r="V5" s="46" t="s">
-        <v>180</v>
-      </c>
-      <c r="W5" s="46" t="s">
-        <v>298</v>
-      </c>
-      <c r="X5" s="46" t="s">
-        <v>299</v>
-      </c>
-      <c r="Y5" s="46" t="s">
-        <v>300</v>
-      </c>
-      <c r="Z5" s="46" t="s">
-        <v>301</v>
-      </c>
-      <c r="AA5" s="46" t="s">
-        <v>302</v>
-      </c>
-      <c r="AB5" s="46" t="s">
-        <v>244</v>
-      </c>
-      <c r="AC5" s="46" t="s">
-        <v>303</v>
-      </c>
-      <c r="AD5" s="46" t="s">
-        <v>304</v>
-      </c>
-      <c r="AE5" s="46" t="s">
-        <v>305</v>
-      </c>
-      <c r="AF5" s="46" t="s">
-        <v>306</v>
-      </c>
-      <c r="AG5" s="46" t="s">
-        <v>307</v>
-      </c>
-      <c r="AH5" s="46" t="s">
-        <v>308</v>
-      </c>
-      <c r="AI5" s="46" t="s">
-        <v>309</v>
-      </c>
-      <c r="AJ5" s="46" t="s">
-        <v>310</v>
-      </c>
-      <c r="AK5" s="46" t="s">
-        <v>311</v>
-      </c>
-      <c r="AL5" s="46" t="s">
-        <v>312</v>
-      </c>
-      <c r="AM5" s="46" t="s">
-        <v>313</v>
-      </c>
-      <c r="AN5" s="46" t="s">
-        <v>314</v>
-      </c>
-      <c r="AO5" s="46" t="s">
-        <v>315</v>
-      </c>
-      <c r="AP5" s="46" t="s">
-        <v>316</v>
-      </c>
-      <c r="AQ5" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="AR5" s="46" t="s">
-        <v>317</v>
-      </c>
-      <c r="AS5" s="46" t="s">
-        <v>318</v>
-      </c>
-      <c r="AT5" s="46" t="s">
-        <v>319</v>
-      </c>
-      <c r="AU5" s="46" t="s">
-        <v>320</v>
-      </c>
-      <c r="AV5" s="46" t="s">
-        <v>263</v>
-      </c>
-      <c r="AW5" s="46" t="s">
-        <v>321</v>
-      </c>
-      <c r="AX5" s="46" t="s">
-        <v>322</v>
-      </c>
-      <c r="AY5" s="46" t="s">
-        <v>323</v>
-      </c>
-      <c r="AZ5" s="46" t="s">
-        <v>324</v>
-      </c>
-      <c r="BA5" s="46" t="s">
-        <v>325</v>
-      </c>
-      <c r="BB5" s="46" t="s">
-        <v>326</v>
-      </c>
-      <c r="BC5" s="46" t="s">
-        <v>327</v>
-      </c>
-      <c r="BD5" s="46" t="s">
-        <v>328</v>
-      </c>
-      <c r="BE5" s="46" t="s">
-        <v>329</v>
-      </c>
-      <c r="BF5" s="46" t="s">
-        <v>330</v>
-      </c>
-      <c r="BG5" s="46" t="s">
-        <v>213</v>
-      </c>
-      <c r="BH5" s="46" t="s">
-        <v>331</v>
-      </c>
-      <c r="BI5" s="46" t="s">
+      <c r="BH5" s="68" t="s">
         <v>332</v>
       </c>
-      <c r="BJ5" s="46" t="s">
+      <c r="BI5" s="68" t="s">
         <v>333</v>
       </c>
-      <c r="BK5" s="46" t="s">
+      <c r="BJ5" s="68" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="6" spans="1:63">
-      <c r="A6" s="46" t="s">
+      <c r="BK5" s="68" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="7" spans="1:63">
-      <c r="A7" s="46" t="s">
+      <c r="BL5" s="68" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:64">
+      <c r="A6" s="68" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="8" spans="1:63">
-      <c r="A8" s="46" t="s">
+    <row r="7" spans="1:64">
+      <c r="A7" s="68" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="9" spans="1:63">
-      <c r="A9" s="46" t="s">
+    <row r="8" spans="1:64">
+      <c r="A8" s="68" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="10" spans="1:63">
-      <c r="A10" s="46" t="s">
+    <row r="9" spans="1:64">
+      <c r="A9" s="68" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="11" spans="1:63">
-      <c r="A11" s="46" t="s">
+    <row r="10" spans="1:64">
+      <c r="A10" s="68" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="12" spans="1:63">
-      <c r="A12" s="46" t="s">
+    <row r="11" spans="1:64">
+      <c r="A11" s="68" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="13" spans="1:63">
-      <c r="A13" s="46" t="s">
+    <row r="12" spans="1:64">
+      <c r="A12" s="68" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="14" spans="1:63">
-      <c r="A14" s="46" t="s">
+    <row r="13" spans="1:64">
+      <c r="A13" s="68" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="15" spans="1:63">
-      <c r="A15" s="46" t="s">
+    <row r="14" spans="1:64">
+      <c r="A14" s="68" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="16" spans="1:63">
-      <c r="A16" s="46" t="s">
+    <row r="15" spans="1:64">
+      <c r="A15" s="68" t="s">
         <v>345</v>
       </c>
     </row>
+    <row r="16" spans="1:64">
+      <c r="A16" s="68" t="s">
+        <v>346</v>
+      </c>
+    </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="46" t="s">
-        <v>346</v>
+      <c r="A17" s="68" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="46" t="s">
-        <v>347</v>
+      <c r="A18" s="68" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="46" t="s">
-        <v>348</v>
+      <c r="A19" s="68" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="46" t="s">
-        <v>349</v>
+      <c r="A20" s="68" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" s="46" t="s">
-        <v>350</v>
+      <c r="A21" s="68" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" s="46" t="s">
-        <v>351</v>
+      <c r="A22" s="68" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" s="46" t="s">
-        <v>352</v>
+      <c r="A23" s="68" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="46" t="s">
-        <v>353</v>
+      <c r="A24" s="68" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="25" spans="1:1">
-      <c r="A25" s="46" t="s">
-        <v>354</v>
+      <c r="A25" s="68" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="26" spans="1:1">
-      <c r="A26" s="46" t="s">
-        <v>355</v>
+      <c r="A26" s="68" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="27" spans="1:1">
-      <c r="A27" s="46" t="s">
-        <v>356</v>
+      <c r="A27" s="68" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="28" spans="1:1">
-      <c r="A28" s="46" t="s">
-        <v>357</v>
+      <c r="A28" s="68" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" s="46" t="s">
-        <v>358</v>
+      <c r="A29" s="68" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="30" spans="1:1">
-      <c r="A30" s="46" t="s">
-        <v>359</v>
+      <c r="A30" s="68" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" s="46" t="s">
-        <v>360</v>
+      <c r="A31" s="68" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" s="46" t="s">
-        <v>361</v>
+      <c r="A32" s="68" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="46" t="s">
-        <v>362</v>
+      <c r="A33" s="68" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="46" t="s">
-        <v>363</v>
+      <c r="A34" s="68" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="46" t="s">
-        <v>364</v>
+      <c r="A35" s="68" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="46" t="s">
-        <v>365</v>
+      <c r="A36" s="68" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="37" spans="1:1">
-      <c r="A37" s="46" t="s">
-        <v>366</v>
+      <c r="A37" s="68" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" s="46" t="s">
-        <v>367</v>
+      <c r="A38" s="68" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" s="46" t="s">
-        <v>368</v>
+      <c r="A39" s="68" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="40" spans="1:1">
-      <c r="A40" s="46" t="s">
-        <v>369</v>
+      <c r="A40" s="68" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="41" spans="1:1">
-      <c r="A41" s="46" t="s">
-        <v>370</v>
+      <c r="A41" s="68" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="46" t="s">
-        <v>371</v>
+      <c r="A42" s="68" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="43" spans="1:1">
-      <c r="A43" s="46" t="s">
-        <v>372</v>
+      <c r="A43" s="68" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="44" spans="1:1">
-      <c r="A44" s="46" t="s">
-        <v>373</v>
+      <c r="A44" s="68" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="45" spans="1:1">
-      <c r="A45" s="46" t="s">
-        <v>374</v>
+      <c r="A45" s="68" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="46" spans="1:1">
-      <c r="A46" s="46" t="s">
-        <v>375</v>
+      <c r="A46" s="68" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="47" spans="1:1">
-      <c r="A47" s="46" t="s">
-        <v>376</v>
+      <c r="A47" s="68" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="46" t="s">
-        <v>377</v>
+      <c r="A48" s="68" t="s">
+        <v>378</v>
       </c>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="46" t="s">
-        <v>378</v>
+      <c r="A49" s="68" t="s">
+        <v>379</v>
       </c>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" s="46" t="s">
-        <v>379</v>
+      <c r="A50" s="68" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="46" t="s">
-        <v>380</v>
+      <c r="A51" s="68" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="52" spans="1:1">
-      <c r="A52" s="46" t="s">
-        <v>381</v>
+      <c r="A52" s="68" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="53" spans="1:1">
-      <c r="A53" s="46" t="s">
-        <v>382</v>
+      <c r="A53" s="68" t="s">
+        <v>383</v>
       </c>
     </row>
     <row r="54" spans="1:1">
-      <c r="A54" s="46" t="s">
-        <v>383</v>
+      <c r="A54" s="68" t="s">
+        <v>384</v>
       </c>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" s="46" t="s">
-        <v>384</v>
+      <c r="A55" s="68" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="56" spans="1:1">
-      <c r="A56" s="46" t="s">
-        <v>385</v>
+      <c r="A56" s="68" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="57" spans="1:1">
-      <c r="A57" s="46" t="s">
-        <v>386</v>
+      <c r="A57" s="68" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="58" spans="1:1">
-      <c r="A58" s="46" t="s">
-        <v>387</v>
+      <c r="A58" s="68" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="59" spans="1:1">
-      <c r="A59" s="46" t="s">
-        <v>388</v>
+      <c r="A59" s="68" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="60" spans="1:1">
-      <c r="A60" s="46" t="s">
-        <v>389</v>
+      <c r="A60" s="68" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="61" spans="1:1">
-      <c r="A61" s="46" t="s">
-        <v>390</v>
+      <c r="A61" s="68" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="62" spans="1:1">
-      <c r="A62" s="46" t="s">
-        <v>391</v>
+      <c r="A62" s="68" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="63" spans="1:1">
-      <c r="A63" s="46" t="s">
-        <v>392</v>
+      <c r="A63" s="68" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="64" spans="1:1">
-      <c r="A64" s="46" t="s">
-        <v>393</v>
+      <c r="A64" s="68" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="65" spans="1:1">
-      <c r="A65" s="46" t="s">
-        <v>394</v>
+      <c r="A65" s="68" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="66" spans="1:1">
-      <c r="A66" s="46" t="s">
-        <v>395</v>
+      <c r="A66" s="68" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="67" spans="1:1">
-      <c r="A67" s="46" t="s">
-        <v>396</v>
+      <c r="A67" s="68" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="68" spans="1:1">
-      <c r="A68" s="46" t="s">
-        <v>397</v>
+      <c r="A68" s="68" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="69" spans="1:1">
-      <c r="A69" s="46" t="s">
-        <v>398</v>
+      <c r="A69" s="68" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="70" spans="1:1">
-      <c r="A70" s="46" t="s">
-        <v>399</v>
+      <c r="A70" s="68" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="71" spans="1:1">
-      <c r="A71" s="46" t="s">
-        <v>400</v>
+      <c r="A71" s="68" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="72" spans="1:1">
-      <c r="A72" s="46" t="s">
-        <v>401</v>
+      <c r="A72" s="68" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="73" spans="1:1">
-      <c r="A73" s="46" t="s">
-        <v>402</v>
+      <c r="A73" s="68" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="74" spans="1:1">
-      <c r="A74" s="46" t="s">
-        <v>403</v>
+      <c r="A74" s="68" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="75" spans="1:1">
-      <c r="A75" s="46" t="s">
-        <v>404</v>
+      <c r="A75" s="68" t="s">
+        <v>405</v>
       </c>
     </row>
     <row r="76" spans="1:1">
-      <c r="A76" s="46" t="s">
-        <v>405</v>
+      <c r="A76" s="68" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="77" spans="1:1">
-      <c r="A77" s="46" t="s">
-        <v>406</v>
+      <c r="A77" s="68" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="78" spans="1:1">
-      <c r="A78" s="46" t="s">
-        <v>407</v>
+      <c r="A78" s="68" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="79" spans="1:1">
-      <c r="A79" s="46" t="s">
-        <v>408</v>
+      <c r="A79" s="68" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="80" spans="1:1">
-      <c r="A80" s="46" t="s">
-        <v>409</v>
+      <c r="A80" s="68" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="81" spans="1:1">
-      <c r="A81" s="46" t="s">
-        <v>410</v>
+      <c r="A81" s="68" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="82" spans="1:1">
-      <c r="A82" s="46" t="s">
-        <v>411</v>
+      <c r="A82" s="68" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="83" spans="1:1">
-      <c r="A83" s="46" t="s">
-        <v>412</v>
+      <c r="A83" s="68" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="84" spans="1:1">
-      <c r="A84" s="46" t="s">
-        <v>413</v>
+      <c r="A84" s="68" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="85" spans="1:1">
-      <c r="A85" s="46" t="s">
-        <v>414</v>
+      <c r="A85" s="68" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="86" spans="1:1">
-      <c r="A86" s="46" t="s">
-        <v>415</v>
+      <c r="A86" s="68" t="s">
+        <v>416</v>
       </c>
     </row>
     <row r="87" spans="1:1">
-      <c r="A87" s="46" t="s">
-        <v>416</v>
+      <c r="A87" s="68" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="88" spans="1:1">
-      <c r="A88" s="46" t="s">
-        <v>417</v>
+      <c r="A88" s="68" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="89" spans="1:1">
-      <c r="A89" s="46" t="s">
-        <v>418</v>
+      <c r="A89" s="68" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="90" spans="1:1">
-      <c r="A90" s="46" t="s">
-        <v>419</v>
+      <c r="A90" s="68" t="s">
+        <v>420</v>
       </c>
     </row>
     <row r="91" spans="1:1">
-      <c r="A91" s="46" t="s">
-        <v>420</v>
+      <c r="A91" s="68" t="s">
+        <v>421</v>
       </c>
     </row>
     <row r="92" spans="1:1">
-      <c r="A92" s="46" t="s">
-        <v>421</v>
+      <c r="A92" s="68" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="93" spans="1:1">
-      <c r="A93" s="46" t="s">
-        <v>422</v>
+      <c r="A93" s="68" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="94" spans="1:1">
-      <c r="A94" s="46" t="s">
-        <v>423</v>
+      <c r="A94" s="68" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="95" spans="1:1">
-      <c r="A95" s="46" t="s">
-        <v>424</v>
+      <c r="A95" s="68" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="96" spans="1:1">
-      <c r="A96" s="46" t="s">
-        <v>425</v>
+      <c r="A96" s="68" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="97" spans="1:1">
-      <c r="A97" s="46" t="s">
-        <v>426</v>
+      <c r="A97" s="68" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="98" spans="1:1">
-      <c r="A98" s="46" t="s">
-        <v>427</v>
+      <c r="A98" s="68" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="99" spans="1:1">
-      <c r="A99" s="46" t="s">
-        <v>428</v>
+      <c r="A99" s="68" t="s">
+        <v>429</v>
       </c>
     </row>
     <row r="100" spans="1:1">
-      <c r="A100" s="46" t="s">
-        <v>429</v>
+      <c r="A100" s="68" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="101" spans="1:1">
-      <c r="A101" s="46" t="s">
-        <v>430</v>
+      <c r="A101" s="68" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="102" spans="1:1">
-      <c r="A102" s="46" t="s">
-        <v>431</v>
+      <c r="A102" s="68" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="103" spans="1:1">
-      <c r="A103" s="46" t="s">
-        <v>432</v>
+      <c r="A103" s="68" t="s">
+        <v>433</v>
       </c>
     </row>
     <row r="104" spans="1:1">
-      <c r="A104" s="46" t="s">
-        <v>433</v>
+      <c r="A104" s="68" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="105" spans="1:1">
-      <c r="A105" s="46" t="s">
-        <v>434</v>
+      <c r="A105" s="68" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="106" spans="1:1">
-      <c r="A106" s="46" t="s">
-        <v>435</v>
+      <c r="A106" s="68" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="107" spans="1:1">
-      <c r="A107" s="46" t="s">
-        <v>436</v>
+      <c r="A107" s="68" t="s">
+        <v>437</v>
       </c>
     </row>
     <row r="108" spans="1:1">
-      <c r="A108" s="46" t="s">
-        <v>437</v>
+      <c r="A108" s="68" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="109" spans="1:1">
-      <c r="A109" s="46" t="s">
-        <v>438</v>
+      <c r="A109" s="68" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="110" spans="1:1">
-      <c r="A110" s="46" t="s">
-        <v>439</v>
+      <c r="A110" s="68" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="111" spans="1:1">
-      <c r="A111" s="46" t="s">
-        <v>440</v>
+      <c r="A111" s="68" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="112" spans="1:1">
-      <c r="A112" s="46" t="s">
-        <v>441</v>
+      <c r="A112" s="68" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="113" spans="1:1">
-      <c r="A113" s="46" t="s">
-        <v>442</v>
+      <c r="A113" s="68" t="s">
+        <v>443</v>
       </c>
     </row>
     <row r="114" spans="1:1">
-      <c r="A114" s="46" t="s">
-        <v>443</v>
+      <c r="A114" s="68" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="115" spans="1:1">
-      <c r="A115" s="46" t="s">
-        <v>444</v>
+      <c r="A115" s="68" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="116" spans="1:1">
-      <c r="A116" s="46" t="s">
-        <v>445</v>
+      <c r="A116" s="68" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="117" spans="1:1">
-      <c r="A117" s="46" t="s">
-        <v>446</v>
+      <c r="A117" s="68" t="s">
+        <v>447</v>
       </c>
     </row>
     <row r="118" spans="1:1">
-      <c r="A118" s="46" t="s">
-        <v>447</v>
+      <c r="A118" s="68" t="s">
+        <v>448</v>
       </c>
     </row>
     <row r="119" spans="1:1">
-      <c r="A119" s="46" t="s">
-        <v>448</v>
+      <c r="A119" s="68" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="120" spans="1:1">
-      <c r="A120" s="46" t="s">
-        <v>449</v>
+      <c r="A120" s="68" t="s">
+        <v>450</v>
       </c>
     </row>
     <row r="121" spans="1:1">
-      <c r="A121" s="46" t="s">
-        <v>450</v>
+      <c r="A121" s="68" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="122" spans="1:1">
-      <c r="A122" s="46" t="s">
-        <v>451</v>
+      <c r="A122" s="68" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="123" spans="1:1">
-      <c r="A123" s="46" t="s">
-        <v>452</v>
+      <c r="A123" s="68" t="s">
+        <v>453</v>
       </c>
     </row>
     <row r="124" spans="1:1">
-      <c r="A124" s="46" t="s">
-        <v>453</v>
+      <c r="A124" s="68" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="125" spans="1:1">
-      <c r="A125" s="46" t="s">
-        <v>454</v>
+      <c r="A125" s="68" t="s">
+        <v>455</v>
       </c>
     </row>
     <row r="126" spans="1:1">
-      <c r="A126" s="46" t="s">
-        <v>455</v>
+      <c r="A126" s="68" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="127" spans="1:1">
-      <c r="A127" s="46" t="s">
-        <v>456</v>
+      <c r="A127" s="68" t="s">
+        <v>457</v>
       </c>
     </row>
     <row r="128" spans="1:1">
-      <c r="A128" s="46" t="s">
-        <v>457</v>
+      <c r="A128" s="68" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="129" spans="1:1">
-      <c r="A129" s="46" t="s">
-        <v>458</v>
+      <c r="A129" s="68" t="s">
+        <v>459</v>
       </c>
     </row>
     <row r="130" spans="1:1">
-      <c r="A130" s="46" t="s">
-        <v>459</v>
+      <c r="A130" s="68" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="131" spans="1:1">
-      <c r="A131" s="46" t="s">
-        <v>460</v>
+      <c r="A131" s="68" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="132" spans="1:1">
-      <c r="A132" s="46" t="s">
-        <v>461</v>
+      <c r="A132" s="68" t="s">
+        <v>462</v>
       </c>
     </row>
     <row r="133" spans="1:1">
-      <c r="A133" s="46" t="s">
-        <v>462</v>
+      <c r="A133" s="68" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="134" spans="1:1">
-      <c r="A134" s="46" t="s">
-        <v>463</v>
+      <c r="A134" s="68" t="s">
+        <v>464</v>
       </c>
     </row>
     <row r="135" spans="1:1">
-      <c r="A135" s="46" t="s">
-        <v>464</v>
+      <c r="A135" s="68" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="136" spans="1:1">
-      <c r="A136" s="46" t="s">
-        <v>465</v>
+      <c r="A136" s="68" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="137" spans="1:1">
-      <c r="A137" s="46" t="s">
-        <v>466</v>
+      <c r="A137" s="68" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="138" spans="1:1">
-      <c r="A138" s="46" t="s">
-        <v>467</v>
+      <c r="A138" s="68" t="s">
+        <v>468</v>
       </c>
     </row>
     <row r="139" spans="1:1">
-      <c r="A139" s="46" t="s">
-        <v>468</v>
+      <c r="A139" s="68" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="140" spans="1:1">
-      <c r="A140" s="46" t="s">
-        <v>469</v>
+      <c r="A140" s="68" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="141" spans="1:1">
-      <c r="A141" s="46" t="s">
-        <v>470</v>
+      <c r="A141" s="68" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="142" spans="1:1">
-      <c r="A142" s="46" t="s">
-        <v>471</v>
+      <c r="A142" s="68" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="143" spans="1:1">
-      <c r="A143" s="46" t="s">
-        <v>472</v>
+      <c r="A143" s="68" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="144" spans="1:1">
-      <c r="A144" s="46" t="s">
-        <v>473</v>
+      <c r="A144" s="68" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="145" spans="1:1">
-      <c r="A145" s="46" t="s">
-        <v>474</v>
+      <c r="A145" s="68" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="146" spans="1:1">
-      <c r="A146" s="46" t="s">
-        <v>475</v>
+      <c r="A146" s="68" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="147" spans="1:1">
-      <c r="A147" s="46" t="s">
-        <v>476</v>
+      <c r="A147" s="68" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="148" spans="1:1">
-      <c r="A148" s="46" t="s">
-        <v>477</v>
+      <c r="A148" s="68" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="149" spans="1:1">
-      <c r="A149" s="46" t="s">
-        <v>478</v>
+      <c r="A149" s="68" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="150" spans="1:1">
-      <c r="A150" s="46" t="s">
-        <v>479</v>
+      <c r="A150" s="68" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="151" spans="1:1">
-      <c r="A151" s="46" t="s">
-        <v>480</v>
+      <c r="A151" s="68" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="152" spans="1:1">
-      <c r="A152" s="46" t="s">
-        <v>481</v>
+      <c r="A152" s="68" t="s">
+        <v>482</v>
       </c>
     </row>
     <row r="153" spans="1:1">
-      <c r="A153" s="46" t="s">
-        <v>482</v>
+      <c r="A153" s="68" t="s">
+        <v>483</v>
       </c>
     </row>
   </sheetData>

</xml_diff>